<commit_message>
Auto commit - 06100928
</commit_message>
<xml_diff>
--- a/IM/202606_Service_Count_Report.xlsx
+++ b/IM/202606_Service_Count_Report.xlsx
@@ -5247,7 +5247,7 @@
         <v>45</v>
       </c>
       <c r="B47" s="7">
-        <v>2026061563</v>
+        <v>2026061564</v>
       </c>
       <c r="C47" s="7">
         <v>1</v>
@@ -5286,7 +5286,7 @@
         <v>218</v>
       </c>
       <c r="O47" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P47" s="7"/>
       <c r="Q47" s="7">
@@ -5295,13 +5295,9 @@
       <c r="R47" s="7">
         <v>15624</v>
       </c>
-      <c r="S47" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S47" s="7"/>
       <c r="T47" s="7"/>
-      <c r="U47" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
       <c r="X47" s="7"/>
@@ -5321,7 +5317,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="3">
-        <v>2026061564</v>
+        <v>2026061563</v>
       </c>
       <c r="C48" s="3">
         <v>1</v>
@@ -5360,7 +5356,7 @@
         <v>218</v>
       </c>
       <c r="O48" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P48" s="3"/>
       <c r="Q48" s="3">
@@ -5369,9 +5365,13 @@
       <c r="R48" s="3">
         <v>15624</v>
       </c>
-      <c r="S48" s="3"/>
+      <c r="S48" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T48" s="3"/>
-      <c r="U48" s="3"/>
+      <c r="U48" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
       <c r="X48" s="3"/>
@@ -6467,7 +6467,7 @@
         <v>63</v>
       </c>
       <c r="B65" s="7">
-        <v>2026060411</v>
+        <v>2026060412</v>
       </c>
       <c r="C65" s="7">
         <v>1</v>
@@ -6506,7 +6506,7 @@
         <v>241</v>
       </c>
       <c r="O65" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P65" s="7"/>
       <c r="Q65" s="7">
@@ -6515,9 +6515,7 @@
       <c r="R65" s="7">
         <v>386927</v>
       </c>
-      <c r="S65" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S65" s="7"/>
       <c r="T65" s="7"/>
       <c r="U65" s="7"/>
       <c r="V65" s="7"/>
@@ -6539,7 +6537,7 @@
         <v>64</v>
       </c>
       <c r="B66" s="3">
-        <v>2026060412</v>
+        <v>2026060411</v>
       </c>
       <c r="C66" s="3">
         <v>1</v>
@@ -6578,7 +6576,7 @@
         <v>241</v>
       </c>
       <c r="O66" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P66" s="3"/>
       <c r="Q66" s="3">
@@ -6587,7 +6585,9 @@
       <c r="R66" s="3">
         <v>386927</v>
       </c>
-      <c r="S66" s="3"/>
+      <c r="S66" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T66" s="3"/>
       <c r="U66" s="3"/>
       <c r="V66" s="3"/>
@@ -6743,7 +6743,7 @@
         <v>67</v>
       </c>
       <c r="B69" s="7">
-        <v>2026060127</v>
+        <v>2026060128</v>
       </c>
       <c r="C69" s="7">
         <v>1</v>
@@ -6782,16 +6782,14 @@
         <v>267</v>
       </c>
       <c r="O69" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P69" s="7"/>
       <c r="Q69" s="7"/>
       <c r="R69" s="7">
         <v>212738</v>
       </c>
-      <c r="S69" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S69" s="7"/>
       <c r="T69" s="7"/>
       <c r="U69" s="7"/>
       <c r="V69" s="7"/>
@@ -6809,7 +6807,7 @@
         <v>68</v>
       </c>
       <c r="B70" s="3">
-        <v>2026060128</v>
+        <v>2026060127</v>
       </c>
       <c r="C70" s="3">
         <v>1</v>
@@ -6848,14 +6846,16 @@
         <v>267</v>
       </c>
       <c r="O70" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P70" s="3"/>
       <c r="Q70" s="3"/>
       <c r="R70" s="3">
         <v>212738</v>
       </c>
-      <c r="S70" s="3"/>
+      <c r="S70" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T70" s="3"/>
       <c r="U70" s="3"/>
       <c r="V70" s="3"/>
@@ -8547,7 +8547,7 @@
         <v>94</v>
       </c>
       <c r="B96" s="3">
-        <v>2026060665</v>
+        <v>2026060664</v>
       </c>
       <c r="C96" s="3">
         <v>1</v>
@@ -8586,7 +8586,7 @@
         <v>353</v>
       </c>
       <c r="O96" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P96" s="3">
         <v>2480</v>
@@ -8597,7 +8597,9 @@
       <c r="R96" s="3">
         <v>11884</v>
       </c>
-      <c r="S96" s="3"/>
+      <c r="S96" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T96" s="3"/>
       <c r="U96" s="3"/>
       <c r="V96" s="3"/>
@@ -8619,7 +8621,7 @@
         <v>95</v>
       </c>
       <c r="B97" s="7">
-        <v>2026060664</v>
+        <v>2026060665</v>
       </c>
       <c r="C97" s="7">
         <v>1</v>
@@ -8658,7 +8660,7 @@
         <v>353</v>
       </c>
       <c r="O97" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P97" s="7">
         <v>2480</v>
@@ -8669,9 +8671,7 @@
       <c r="R97" s="7">
         <v>11884</v>
       </c>
-      <c r="S97" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S97" s="7"/>
       <c r="T97" s="7"/>
       <c r="U97" s="7"/>
       <c r="V97" s="7"/>
@@ -10421,7 +10421,7 @@
         <v>121</v>
       </c>
       <c r="B123" s="7">
-        <v>2026061104</v>
+        <v>2026061103</v>
       </c>
       <c r="C123" s="7">
         <v>1</v>
@@ -10458,14 +10458,16 @@
       </c>
       <c r="N123" s="8"/>
       <c r="O123" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P123" s="7"/>
       <c r="Q123" s="7"/>
       <c r="R123" s="7">
         <v>66000</v>
       </c>
-      <c r="S123" s="7"/>
+      <c r="S123" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T123" s="7"/>
       <c r="U123" s="7"/>
       <c r="V123" s="7"/>
@@ -10487,7 +10489,7 @@
         <v>122</v>
       </c>
       <c r="B124" s="3">
-        <v>2026061103</v>
+        <v>2026061104</v>
       </c>
       <c r="C124" s="3">
         <v>1</v>
@@ -10524,16 +10526,14 @@
       </c>
       <c r="N124" s="6"/>
       <c r="O124" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P124" s="3"/>
       <c r="Q124" s="3"/>
       <c r="R124" s="3">
         <v>66000</v>
       </c>
-      <c r="S124" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S124" s="3"/>
       <c r="T124" s="3"/>
       <c r="U124" s="3"/>
       <c r="V124" s="3"/>
@@ -10623,7 +10623,7 @@
         <v>124</v>
       </c>
       <c r="B126" s="3">
-        <v>2026060053</v>
+        <v>2026060052</v>
       </c>
       <c r="C126" s="3">
         <v>1</v>
@@ -10662,14 +10662,16 @@
         <v>406</v>
       </c>
       <c r="O126" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P126" s="3"/>
       <c r="Q126" s="3"/>
       <c r="R126" s="3">
         <v>29640</v>
       </c>
-      <c r="S126" s="3"/>
+      <c r="S126" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T126" s="3"/>
       <c r="U126" s="3"/>
       <c r="V126" s="3"/>
@@ -10691,7 +10693,7 @@
         <v>125</v>
       </c>
       <c r="B127" s="7">
-        <v>2026060052</v>
+        <v>2026060053</v>
       </c>
       <c r="C127" s="7">
         <v>1</v>
@@ -10730,16 +10732,14 @@
         <v>406</v>
       </c>
       <c r="O127" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P127" s="7"/>
       <c r="Q127" s="7"/>
       <c r="R127" s="7">
         <v>29640</v>
       </c>
-      <c r="S127" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S127" s="7"/>
       <c r="T127" s="7"/>
       <c r="U127" s="7"/>
       <c r="V127" s="7"/>
@@ -12251,7 +12251,7 @@
         <v>148</v>
       </c>
       <c r="B150" s="3">
-        <v>2026060049</v>
+        <v>2026060048</v>
       </c>
       <c r="C150" s="3">
         <v>1</v>
@@ -12290,14 +12290,16 @@
         <v>438</v>
       </c>
       <c r="O150" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P150" s="3"/>
       <c r="Q150" s="3"/>
       <c r="R150" s="3">
         <v>5766</v>
       </c>
-      <c r="S150" s="3"/>
+      <c r="S150" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T150" s="3"/>
       <c r="U150" s="3"/>
       <c r="V150" s="3"/>
@@ -12319,7 +12321,7 @@
         <v>149</v>
       </c>
       <c r="B151" s="7">
-        <v>2026060048</v>
+        <v>2026060049</v>
       </c>
       <c r="C151" s="7">
         <v>1</v>
@@ -12358,16 +12360,14 @@
         <v>438</v>
       </c>
       <c r="O151" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P151" s="7"/>
       <c r="Q151" s="7"/>
       <c r="R151" s="7">
         <v>5766</v>
       </c>
-      <c r="S151" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S151" s="7"/>
       <c r="T151" s="7"/>
       <c r="U151" s="7"/>
       <c r="V151" s="7"/>
@@ -12727,7 +12727,7 @@
         <v>155</v>
       </c>
       <c r="B157" s="7">
-        <v>2026060526</v>
+        <v>2026060527</v>
       </c>
       <c r="C157" s="7">
         <v>1</v>
@@ -12766,16 +12766,14 @@
         <v>448</v>
       </c>
       <c r="O157" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P157" s="7"/>
       <c r="Q157" s="7"/>
       <c r="R157" s="7">
         <v>33686</v>
       </c>
-      <c r="S157" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S157" s="7"/>
       <c r="T157" s="7"/>
       <c r="U157" s="7"/>
       <c r="V157" s="7"/>
@@ -12785,15 +12783,19 @@
       <c r="Z157" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="AA157" s="7"/>
-      <c r="AB157" s="7"/>
+      <c r="AA157" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB157" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="158" spans="1:28">
       <c r="A158" s="3">
         <v>156</v>
       </c>
       <c r="B158" s="3">
-        <v>2026060527</v>
+        <v>2026060526</v>
       </c>
       <c r="C158" s="3">
         <v>1</v>
@@ -12832,14 +12834,16 @@
         <v>448</v>
       </c>
       <c r="O158" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P158" s="3"/>
       <c r="Q158" s="3"/>
       <c r="R158" s="3">
         <v>33686</v>
       </c>
-      <c r="S158" s="3"/>
+      <c r="S158" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T158" s="3"/>
       <c r="U158" s="3"/>
       <c r="V158" s="3"/>
@@ -12849,9 +12853,7 @@
       <c r="Z158" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="AA158" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA158" s="3"/>
       <c r="AB158" s="3"/>
     </row>
     <row r="159" spans="1:28">
@@ -15089,7 +15091,7 @@
         <v>190</v>
       </c>
       <c r="B192" s="3">
-        <v>2026061260</v>
+        <v>2026061529</v>
       </c>
       <c r="C192" s="3">
         <v>1</v>
@@ -15112,12 +15114,8 @@
       <c r="I192" s="3" t="s">
         <v>519</v>
       </c>
-      <c r="J192" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="K192" s="3" t="s">
-        <v>197</v>
-      </c>
+      <c r="J192" s="3"/>
+      <c r="K192" s="3"/>
       <c r="L192" s="6" t="s">
         <v>167</v>
       </c>
@@ -15128,14 +15126,16 @@
         <v>521</v>
       </c>
       <c r="O192" s="3" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="P192" s="3"/>
       <c r="Q192" s="3"/>
       <c r="R192" s="3">
         <v>0</v>
       </c>
-      <c r="S192" s="3"/>
+      <c r="S192" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T192" s="3"/>
       <c r="U192" s="3"/>
       <c r="V192" s="3"/>
@@ -15143,7 +15143,7 @@
       <c r="X192" s="3"/>
       <c r="Y192" s="3"/>
       <c r="Z192" s="6" t="s">
-        <v>522</v>
+        <v>181</v>
       </c>
       <c r="AA192" s="3" t="s">
         <v>40</v>
@@ -15157,7 +15157,7 @@
         <v>191</v>
       </c>
       <c r="B193" s="7">
-        <v>2026061529</v>
+        <v>2026061260</v>
       </c>
       <c r="C193" s="7">
         <v>1</v>
@@ -15180,8 +15180,12 @@
       <c r="I193" s="7" t="s">
         <v>519</v>
       </c>
-      <c r="J193" s="7"/>
-      <c r="K193" s="7"/>
+      <c r="J193" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="K193" s="7" t="s">
+        <v>197</v>
+      </c>
       <c r="L193" s="8" t="s">
         <v>167</v>
       </c>
@@ -15192,16 +15196,14 @@
         <v>521</v>
       </c>
       <c r="O193" s="7" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="P193" s="7"/>
       <c r="Q193" s="7"/>
       <c r="R193" s="7">
         <v>0</v>
       </c>
-      <c r="S193" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S193" s="7"/>
       <c r="T193" s="7"/>
       <c r="U193" s="7"/>
       <c r="V193" s="7"/>
@@ -15209,7 +15211,7 @@
       <c r="X193" s="7"/>
       <c r="Y193" s="7"/>
       <c r="Z193" s="8" t="s">
-        <v>181</v>
+        <v>522</v>
       </c>
       <c r="AA193" s="7" t="s">
         <v>40</v>
@@ -15221,7 +15223,7 @@
         <v>192</v>
       </c>
       <c r="B194" s="3">
-        <v>2026060475</v>
+        <v>2026060149</v>
       </c>
       <c r="C194" s="3">
         <v>1</v>
@@ -15244,8 +15246,12 @@
       <c r="I194" s="3" t="s">
         <v>524</v>
       </c>
-      <c r="J194" s="3"/>
-      <c r="K194" s="3"/>
+      <c r="J194" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="K194" s="3" t="s">
+        <v>197</v>
+      </c>
       <c r="L194" s="6" t="s">
         <v>167</v>
       </c>
@@ -15256,16 +15262,14 @@
         <v>526</v>
       </c>
       <c r="O194" s="3" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="P194" s="3"/>
       <c r="Q194" s="3"/>
       <c r="R194" s="3">
         <v>0</v>
       </c>
-      <c r="S194" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S194" s="3"/>
       <c r="T194" s="3"/>
       <c r="U194" s="3"/>
       <c r="V194" s="3"/>
@@ -15273,7 +15277,7 @@
       <c r="X194" s="3"/>
       <c r="Y194" s="3"/>
       <c r="Z194" s="6" t="s">
-        <v>181</v>
+        <v>527</v>
       </c>
       <c r="AA194" s="3" t="s">
         <v>40</v>
@@ -15287,7 +15291,7 @@
         <v>193</v>
       </c>
       <c r="B195" s="7">
-        <v>2026060149</v>
+        <v>2026060475</v>
       </c>
       <c r="C195" s="7">
         <v>1</v>
@@ -15310,12 +15314,8 @@
       <c r="I195" s="7" t="s">
         <v>524</v>
       </c>
-      <c r="J195" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="K195" s="7" t="s">
-        <v>197</v>
-      </c>
+      <c r="J195" s="7"/>
+      <c r="K195" s="7"/>
       <c r="L195" s="8" t="s">
         <v>167</v>
       </c>
@@ -15326,14 +15326,16 @@
         <v>526</v>
       </c>
       <c r="O195" s="7" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="P195" s="7"/>
       <c r="Q195" s="7"/>
       <c r="R195" s="7">
         <v>0</v>
       </c>
-      <c r="S195" s="7"/>
+      <c r="S195" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T195" s="7"/>
       <c r="U195" s="7"/>
       <c r="V195" s="7"/>
@@ -15341,7 +15343,7 @@
       <c r="X195" s="7"/>
       <c r="Y195" s="7"/>
       <c r="Z195" s="8" t="s">
-        <v>527</v>
+        <v>181</v>
       </c>
       <c r="AA195" s="7" t="s">
         <v>40</v>
@@ -15583,7 +15585,7 @@
         <v>546</v>
       </c>
       <c r="AB199" s="9">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto commit - 06101128
</commit_message>
<xml_diff>
--- a/IM/202606_Service_Count_Report.xlsx
+++ b/IM/202606_Service_Count_Report.xlsx
@@ -11,14 +11,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Report'!$1:$2</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AA$199</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Report'!$A$1:$AA$200</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="547">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="549">
   <si>
     <t>服務次數統計表        篩選月份：202606</t>
   </si>
@@ -1294,6 +1294,12 @@
   </si>
   <si>
     <t>走道</t>
+  </si>
+  <si>
+    <t>2026-06-10</t>
+  </si>
+  <si>
+    <t>多台卡機無法使用 確認為伺服器設定問題</t>
   </si>
   <si>
     <t>T302800154</t>
@@ -2105,7 +2111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB199"/>
+  <dimension ref="A1:AB200"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
@@ -4969,7 +4975,7 @@
         <v>41</v>
       </c>
       <c r="B43" s="7">
-        <v>2026060673</v>
+        <v>2026060674</v>
       </c>
       <c r="C43" s="7">
         <v>1</v>
@@ -5008,7 +5014,7 @@
         <v>207</v>
       </c>
       <c r="O43" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P43" s="7">
         <v>7927</v>
@@ -5019,9 +5025,7 @@
       <c r="R43" s="7">
         <v>25584</v>
       </c>
-      <c r="S43" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S43" s="7"/>
       <c r="T43" s="7"/>
       <c r="U43" s="7"/>
       <c r="V43" s="7"/>
@@ -5043,7 +5047,7 @@
         <v>42</v>
       </c>
       <c r="B44" s="3">
-        <v>2026060674</v>
+        <v>2026060673</v>
       </c>
       <c r="C44" s="3">
         <v>1</v>
@@ -5082,7 +5086,7 @@
         <v>207</v>
       </c>
       <c r="O44" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P44" s="3">
         <v>7927</v>
@@ -5093,7 +5097,9 @@
       <c r="R44" s="3">
         <v>25584</v>
       </c>
-      <c r="S44" s="3"/>
+      <c r="S44" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T44" s="3"/>
       <c r="U44" s="3"/>
       <c r="V44" s="3"/>
@@ -5247,7 +5253,7 @@
         <v>45</v>
       </c>
       <c r="B47" s="7">
-        <v>2026061564</v>
+        <v>2026061563</v>
       </c>
       <c r="C47" s="7">
         <v>1</v>
@@ -5286,7 +5292,7 @@
         <v>218</v>
       </c>
       <c r="O47" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P47" s="7"/>
       <c r="Q47" s="7">
@@ -5295,9 +5301,13 @@
       <c r="R47" s="7">
         <v>15624</v>
       </c>
-      <c r="S47" s="7"/>
+      <c r="S47" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T47" s="7"/>
-      <c r="U47" s="7"/>
+      <c r="U47" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
       <c r="X47" s="7"/>
@@ -5317,7 +5327,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="3">
-        <v>2026061563</v>
+        <v>2026061564</v>
       </c>
       <c r="C48" s="3">
         <v>1</v>
@@ -5356,7 +5366,7 @@
         <v>218</v>
       </c>
       <c r="O48" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P48" s="3"/>
       <c r="Q48" s="3">
@@ -5365,13 +5375,9 @@
       <c r="R48" s="3">
         <v>15624</v>
       </c>
-      <c r="S48" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S48" s="3"/>
       <c r="T48" s="3"/>
-      <c r="U48" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="U48" s="3"/>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
       <c r="X48" s="3"/>
@@ -5999,7 +6005,7 @@
         <v>56</v>
       </c>
       <c r="B58" s="3">
-        <v>2026060378</v>
+        <v>2026060379</v>
       </c>
       <c r="C58" s="3">
         <v>1</v>
@@ -6036,16 +6042,14 @@
       </c>
       <c r="N58" s="6"/>
       <c r="O58" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P58" s="3"/>
       <c r="Q58" s="3"/>
       <c r="R58" s="3">
         <v>36400</v>
       </c>
-      <c r="S58" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S58" s="3"/>
       <c r="T58" s="3"/>
       <c r="U58" s="3"/>
       <c r="V58" s="3"/>
@@ -6067,7 +6071,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="7">
-        <v>2026060379</v>
+        <v>2026060378</v>
       </c>
       <c r="C59" s="7">
         <v>1</v>
@@ -6104,14 +6108,16 @@
       </c>
       <c r="N59" s="8"/>
       <c r="O59" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P59" s="7"/>
       <c r="Q59" s="7"/>
       <c r="R59" s="7">
         <v>36400</v>
       </c>
-      <c r="S59" s="7"/>
+      <c r="S59" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T59" s="7"/>
       <c r="U59" s="7"/>
       <c r="V59" s="7"/>
@@ -6467,7 +6473,7 @@
         <v>63</v>
       </c>
       <c r="B65" s="7">
-        <v>2026060412</v>
+        <v>2026060411</v>
       </c>
       <c r="C65" s="7">
         <v>1</v>
@@ -6506,7 +6512,7 @@
         <v>241</v>
       </c>
       <c r="O65" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P65" s="7"/>
       <c r="Q65" s="7">
@@ -6515,7 +6521,9 @@
       <c r="R65" s="7">
         <v>386927</v>
       </c>
-      <c r="S65" s="7"/>
+      <c r="S65" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T65" s="7"/>
       <c r="U65" s="7"/>
       <c r="V65" s="7"/>
@@ -6537,7 +6545,7 @@
         <v>64</v>
       </c>
       <c r="B66" s="3">
-        <v>2026060411</v>
+        <v>2026060412</v>
       </c>
       <c r="C66" s="3">
         <v>1</v>
@@ -6576,7 +6584,7 @@
         <v>241</v>
       </c>
       <c r="O66" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P66" s="3"/>
       <c r="Q66" s="3">
@@ -6585,9 +6593,7 @@
       <c r="R66" s="3">
         <v>386927</v>
       </c>
-      <c r="S66" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S66" s="3"/>
       <c r="T66" s="3"/>
       <c r="U66" s="3"/>
       <c r="V66" s="3"/>
@@ -6743,7 +6749,7 @@
         <v>67</v>
       </c>
       <c r="B69" s="7">
-        <v>2026060128</v>
+        <v>2026060127</v>
       </c>
       <c r="C69" s="7">
         <v>1</v>
@@ -6782,14 +6788,16 @@
         <v>267</v>
       </c>
       <c r="O69" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P69" s="7"/>
       <c r="Q69" s="7"/>
       <c r="R69" s="7">
         <v>212738</v>
       </c>
-      <c r="S69" s="7"/>
+      <c r="S69" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T69" s="7"/>
       <c r="U69" s="7"/>
       <c r="V69" s="7"/>
@@ -6807,7 +6815,7 @@
         <v>68</v>
       </c>
       <c r="B70" s="3">
-        <v>2026060127</v>
+        <v>2026060128</v>
       </c>
       <c r="C70" s="3">
         <v>1</v>
@@ -6846,16 +6854,14 @@
         <v>267</v>
       </c>
       <c r="O70" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P70" s="3"/>
       <c r="Q70" s="3"/>
       <c r="R70" s="3">
         <v>212738</v>
       </c>
-      <c r="S70" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S70" s="3"/>
       <c r="T70" s="3"/>
       <c r="U70" s="3"/>
       <c r="V70" s="3"/>
@@ -6873,7 +6879,7 @@
         <v>69</v>
       </c>
       <c r="B71" s="7">
-        <v>2026061436</v>
+        <v>2026061437</v>
       </c>
       <c r="C71" s="7">
         <v>1</v>
@@ -6912,7 +6918,7 @@
         <v>271</v>
       </c>
       <c r="O71" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P71" s="7"/>
       <c r="Q71" s="7">
@@ -6921,9 +6927,7 @@
       <c r="R71" s="7">
         <v>221294</v>
       </c>
-      <c r="S71" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S71" s="7"/>
       <c r="T71" s="7"/>
       <c r="U71" s="7"/>
       <c r="V71" s="7"/>
@@ -6941,7 +6945,7 @@
         <v>70</v>
       </c>
       <c r="B72" s="3">
-        <v>2026061437</v>
+        <v>2026061436</v>
       </c>
       <c r="C72" s="3">
         <v>1</v>
@@ -6980,7 +6984,7 @@
         <v>271</v>
       </c>
       <c r="O72" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P72" s="3"/>
       <c r="Q72" s="3">
@@ -6989,7 +6993,9 @@
       <c r="R72" s="3">
         <v>221294</v>
       </c>
-      <c r="S72" s="3"/>
+      <c r="S72" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T72" s="3"/>
       <c r="U72" s="3"/>
       <c r="V72" s="3"/>
@@ -9739,7 +9745,7 @@
         <v>111</v>
       </c>
       <c r="B113" s="7">
-        <v>2026061006</v>
+        <v>2026061007</v>
       </c>
       <c r="C113" s="7">
         <v>1</v>
@@ -9778,16 +9784,14 @@
         <v>383</v>
       </c>
       <c r="O113" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P113" s="7"/>
       <c r="Q113" s="7"/>
       <c r="R113" s="7">
         <v>57995</v>
       </c>
-      <c r="S113" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S113" s="7"/>
       <c r="T113" s="7"/>
       <c r="U113" s="7"/>
       <c r="V113" s="7"/>
@@ -9809,7 +9813,7 @@
         <v>112</v>
       </c>
       <c r="B114" s="3">
-        <v>2026061007</v>
+        <v>2026061006</v>
       </c>
       <c r="C114" s="3">
         <v>1</v>
@@ -9848,14 +9852,16 @@
         <v>383</v>
       </c>
       <c r="O114" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P114" s="3"/>
       <c r="Q114" s="3"/>
       <c r="R114" s="3">
         <v>57995</v>
       </c>
-      <c r="S114" s="3"/>
+      <c r="S114" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T114" s="3"/>
       <c r="U114" s="3"/>
       <c r="V114" s="3"/>
@@ -11443,7 +11449,7 @@
         <v>136</v>
       </c>
       <c r="B138" s="3">
-        <v>2026060040</v>
+        <v>2026061645</v>
       </c>
       <c r="C138" s="3">
         <v>1</v>
@@ -11455,16 +11461,16 @@
         <v>345</v>
       </c>
       <c r="F138" s="3" t="s">
-        <v>209</v>
+        <v>417</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="H138" s="3" t="s">
-        <v>354</v>
+        <v>137</v>
       </c>
       <c r="I138" s="3" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="J138" s="3" t="s">
         <v>117</v>
@@ -11476,22 +11482,20 @@
         <v>377</v>
       </c>
       <c r="M138" s="6" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="N138" s="6" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="O138" s="3" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="P138" s="3"/>
       <c r="Q138" s="3"/>
       <c r="R138" s="3">
-        <v>29640</v>
-      </c>
-      <c r="S138" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>45926</v>
+      </c>
+      <c r="S138" s="3"/>
       <c r="T138" s="3"/>
       <c r="U138" s="3"/>
       <c r="V138" s="3"/>
@@ -11499,7 +11503,7 @@
       <c r="X138" s="3"/>
       <c r="Y138" s="3"/>
       <c r="Z138" s="6" t="s">
-        <v>349</v>
+        <v>418</v>
       </c>
       <c r="AA138" s="3" t="s">
         <v>40</v>
@@ -11513,7 +11517,7 @@
         <v>137</v>
       </c>
       <c r="B139" s="7">
-        <v>2026060041</v>
+        <v>2026060040</v>
       </c>
       <c r="C139" s="7">
         <v>1</v>
@@ -11534,7 +11538,7 @@
         <v>354</v>
       </c>
       <c r="I139" s="7" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="J139" s="7" t="s">
         <v>117</v>
@@ -11546,20 +11550,22 @@
         <v>377</v>
       </c>
       <c r="M139" s="8" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="N139" s="8" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="O139" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P139" s="7"/>
       <c r="Q139" s="7"/>
       <c r="R139" s="7">
         <v>29640</v>
       </c>
-      <c r="S139" s="7"/>
+      <c r="S139" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T139" s="7"/>
       <c r="U139" s="7"/>
       <c r="V139" s="7"/>
@@ -11572,14 +11578,16 @@
       <c r="AA139" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB139" s="7"/>
+      <c r="AB139" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="140" spans="1:28">
       <c r="A140" s="3">
         <v>138</v>
       </c>
       <c r="B140" s="3">
-        <v>2026060044</v>
+        <v>2026060041</v>
       </c>
       <c r="C140" s="3">
         <v>1</v>
@@ -11594,13 +11602,13 @@
         <v>209</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>202</v>
+        <v>359</v>
       </c>
       <c r="H140" s="3" t="s">
-        <v>50</v>
+        <v>354</v>
       </c>
       <c r="I140" s="3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="J140" s="3" t="s">
         <v>117</v>
@@ -11612,22 +11620,20 @@
         <v>377</v>
       </c>
       <c r="M140" s="6" t="s">
+        <v>420</v>
+      </c>
+      <c r="N140" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="N140" s="6" t="s">
-        <v>422</v>
-      </c>
       <c r="O140" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P140" s="3"/>
       <c r="Q140" s="3"/>
       <c r="R140" s="3">
-        <v>34235</v>
-      </c>
-      <c r="S140" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>29640</v>
+      </c>
+      <c r="S140" s="3"/>
       <c r="T140" s="3"/>
       <c r="U140" s="3"/>
       <c r="V140" s="3"/>
@@ -11640,16 +11646,14 @@
       <c r="AA140" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB140" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB140" s="3"/>
     </row>
     <row r="141" spans="1:28">
       <c r="A141" s="7">
         <v>139</v>
       </c>
       <c r="B141" s="7">
-        <v>2026060045</v>
+        <v>2026060044</v>
       </c>
       <c r="C141" s="7">
         <v>1</v>
@@ -11670,7 +11674,7 @@
         <v>50</v>
       </c>
       <c r="I141" s="7" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="J141" s="7" t="s">
         <v>117</v>
@@ -11682,20 +11686,22 @@
         <v>377</v>
       </c>
       <c r="M141" s="8" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="N141" s="8" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="O141" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P141" s="7"/>
       <c r="Q141" s="7"/>
       <c r="R141" s="7">
         <v>34235</v>
       </c>
-      <c r="S141" s="7"/>
+      <c r="S141" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T141" s="7"/>
       <c r="U141" s="7"/>
       <c r="V141" s="7"/>
@@ -11708,14 +11714,16 @@
       <c r="AA141" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB141" s="7"/>
+      <c r="AB141" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="142" spans="1:28">
       <c r="A142" s="3">
         <v>140</v>
       </c>
       <c r="B142" s="3">
-        <v>2026060042</v>
+        <v>2026060045</v>
       </c>
       <c r="C142" s="3">
         <v>1</v>
@@ -11730,13 +11738,13 @@
         <v>209</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>354</v>
+        <v>202</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>202</v>
+        <v>50</v>
       </c>
       <c r="I142" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J142" s="3" t="s">
         <v>117</v>
@@ -11748,22 +11756,20 @@
         <v>377</v>
       </c>
       <c r="M142" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="N142" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="N142" s="6" t="s">
-        <v>370</v>
-      </c>
       <c r="O142" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P142" s="3"/>
       <c r="Q142" s="3"/>
       <c r="R142" s="3">
-        <v>17791</v>
-      </c>
-      <c r="S142" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>34235</v>
+      </c>
+      <c r="S142" s="3"/>
       <c r="T142" s="3"/>
       <c r="U142" s="3"/>
       <c r="V142" s="3"/>
@@ -11776,16 +11782,14 @@
       <c r="AA142" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB142" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB142" s="3"/>
     </row>
     <row r="143" spans="1:28">
       <c r="A143" s="7">
         <v>141</v>
       </c>
       <c r="B143" s="7">
-        <v>2026060043</v>
+        <v>2026060042</v>
       </c>
       <c r="C143" s="7">
         <v>1</v>
@@ -11806,7 +11810,7 @@
         <v>202</v>
       </c>
       <c r="I143" s="7" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="J143" s="7" t="s">
         <v>117</v>
@@ -11818,20 +11822,22 @@
         <v>377</v>
       </c>
       <c r="M143" s="8" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="N143" s="8" t="s">
         <v>370</v>
       </c>
       <c r="O143" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P143" s="7"/>
       <c r="Q143" s="7"/>
       <c r="R143" s="7">
         <v>17791</v>
       </c>
-      <c r="S143" s="7"/>
+      <c r="S143" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T143" s="7"/>
       <c r="U143" s="7"/>
       <c r="V143" s="7"/>
@@ -11844,14 +11850,16 @@
       <c r="AA143" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB143" s="7"/>
+      <c r="AB143" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="144" spans="1:28">
       <c r="A144" s="3">
         <v>142</v>
       </c>
       <c r="B144" s="3">
-        <v>2026060385</v>
+        <v>2026060043</v>
       </c>
       <c r="C144" s="3">
         <v>1</v>
@@ -11863,43 +11871,41 @@
         <v>345</v>
       </c>
       <c r="F144" s="3" t="s">
-        <v>49</v>
+        <v>209</v>
       </c>
       <c r="G144" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="H144" s="3" t="s">
         <v>202</v>
-      </c>
-      <c r="H144" s="3" t="s">
-        <v>50</v>
       </c>
       <c r="I144" s="3" t="s">
         <v>425</v>
       </c>
       <c r="J144" s="3" t="s">
-        <v>426</v>
+        <v>117</v>
       </c>
       <c r="K144" s="3" t="s">
         <v>36</v>
       </c>
       <c r="L144" s="6" t="s">
-        <v>427</v>
+        <v>377</v>
       </c>
       <c r="M144" s="6" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="N144" s="6" t="s">
-        <v>429</v>
+        <v>370</v>
       </c>
       <c r="O144" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P144" s="3"/>
       <c r="Q144" s="3"/>
       <c r="R144" s="3">
-        <v>122434</v>
-      </c>
-      <c r="S144" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>17791</v>
+      </c>
+      <c r="S144" s="3"/>
       <c r="T144" s="3"/>
       <c r="U144" s="3"/>
       <c r="V144" s="3"/>
@@ -11909,7 +11915,9 @@
       <c r="Z144" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="AA144" s="3"/>
+      <c r="AA144" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="AB144" s="3"/>
     </row>
     <row r="145" spans="1:28">
@@ -11938,22 +11946,22 @@
         <v>50</v>
       </c>
       <c r="I145" s="7" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="J145" s="7" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="K145" s="7" t="s">
         <v>36</v>
       </c>
       <c r="L145" s="8" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M145" s="8" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="N145" s="8" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="O145" s="7" t="s">
         <v>60</v>
@@ -11976,14 +11984,16 @@
       <c r="AA145" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB145" s="7"/>
+      <c r="AB145" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="146" spans="1:28">
       <c r="A146" s="3">
         <v>144</v>
       </c>
       <c r="B146" s="3">
-        <v>2026061412</v>
+        <v>2026060385</v>
       </c>
       <c r="C146" s="3">
         <v>1</v>
@@ -11995,31 +12005,31 @@
         <v>345</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="G146" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="H146" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="H146" s="3" t="s">
-        <v>137</v>
-      </c>
       <c r="I146" s="3" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="J146" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="K146" s="3" t="s">
         <v>36</v>
       </c>
       <c r="L146" s="6" t="s">
-        <v>373</v>
+        <v>429</v>
       </c>
       <c r="M146" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="N146" s="6" t="s">
         <v>431</v>
-      </c>
-      <c r="N146" s="6" t="s">
-        <v>432</v>
       </c>
       <c r="O146" s="3" t="s">
         <v>39</v>
@@ -12027,7 +12037,7 @@
       <c r="P146" s="3"/>
       <c r="Q146" s="3"/>
       <c r="R146" s="3">
-        <v>13563</v>
+        <v>122434</v>
       </c>
       <c r="S146" s="3" t="s">
         <v>40</v>
@@ -12049,7 +12059,7 @@
         <v>145</v>
       </c>
       <c r="B147" s="7">
-        <v>2026061413</v>
+        <v>2026061412</v>
       </c>
       <c r="C147" s="7">
         <v>1</v>
@@ -12070,10 +12080,10 @@
         <v>137</v>
       </c>
       <c r="I147" s="7" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="J147" s="7" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="K147" s="7" t="s">
         <v>36</v>
@@ -12082,20 +12092,22 @@
         <v>373</v>
       </c>
       <c r="M147" s="8" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="N147" s="8" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="O147" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P147" s="7"/>
       <c r="Q147" s="7"/>
       <c r="R147" s="7">
         <v>13563</v>
       </c>
-      <c r="S147" s="7"/>
+      <c r="S147" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T147" s="7"/>
       <c r="U147" s="7"/>
       <c r="V147" s="7"/>
@@ -12105,9 +12117,7 @@
       <c r="Z147" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="AA147" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA147" s="7"/>
       <c r="AB147" s="7"/>
     </row>
     <row r="148" spans="1:28">
@@ -12115,7 +12125,7 @@
         <v>146</v>
       </c>
       <c r="B148" s="3">
-        <v>2026060061</v>
+        <v>2026061413</v>
       </c>
       <c r="C148" s="3">
         <v>1</v>
@@ -12127,43 +12137,41 @@
         <v>345</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>209</v>
+        <v>31</v>
       </c>
       <c r="G148" s="3" t="s">
-        <v>257</v>
+        <v>50</v>
       </c>
       <c r="H148" s="3" t="s">
-        <v>70</v>
+        <v>137</v>
       </c>
       <c r="I148" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="J148" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="K148" s="3" t="s">
         <v>36</v>
       </c>
       <c r="L148" s="6" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="M148" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="N148" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="N148" s="6" t="s">
-        <v>435</v>
-      </c>
       <c r="O148" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P148" s="3"/>
       <c r="Q148" s="3"/>
       <c r="R148" s="3">
-        <v>702</v>
-      </c>
-      <c r="S148" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>13563</v>
+      </c>
+      <c r="S148" s="3"/>
       <c r="T148" s="3"/>
       <c r="U148" s="3"/>
       <c r="V148" s="3"/>
@@ -12176,16 +12184,14 @@
       <c r="AA148" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB148" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB148" s="3"/>
     </row>
     <row r="149" spans="1:28">
       <c r="A149" s="7">
         <v>147</v>
       </c>
       <c r="B149" s="7">
-        <v>2026060062</v>
+        <v>2026060061</v>
       </c>
       <c r="C149" s="7">
         <v>1</v>
@@ -12206,10 +12212,10 @@
         <v>70</v>
       </c>
       <c r="I149" s="7" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="J149" s="7" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="K149" s="7" t="s">
         <v>36</v>
@@ -12218,20 +12224,22 @@
         <v>377</v>
       </c>
       <c r="M149" s="8" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="N149" s="8" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="O149" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P149" s="7"/>
       <c r="Q149" s="7"/>
       <c r="R149" s="7">
         <v>702</v>
       </c>
-      <c r="S149" s="7"/>
+      <c r="S149" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T149" s="7"/>
       <c r="U149" s="7"/>
       <c r="V149" s="7"/>
@@ -12244,14 +12252,16 @@
       <c r="AA149" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB149" s="7"/>
+      <c r="AB149" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="150" spans="1:28">
       <c r="A150" s="3">
         <v>148</v>
       </c>
       <c r="B150" s="3">
-        <v>2026060048</v>
+        <v>2026060062</v>
       </c>
       <c r="C150" s="3">
         <v>1</v>
@@ -12266,16 +12276,16 @@
         <v>209</v>
       </c>
       <c r="G150" s="3" t="s">
-        <v>137</v>
+        <v>257</v>
       </c>
       <c r="H150" s="3" t="s">
-        <v>106</v>
+        <v>70</v>
       </c>
       <c r="I150" s="3" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="J150" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="K150" s="3" t="s">
         <v>36</v>
@@ -12284,22 +12294,20 @@
         <v>377</v>
       </c>
       <c r="M150" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="N150" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="N150" s="6" t="s">
-        <v>438</v>
-      </c>
       <c r="O150" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P150" s="3"/>
       <c r="Q150" s="3"/>
       <c r="R150" s="3">
-        <v>5766</v>
-      </c>
-      <c r="S150" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>702</v>
+      </c>
+      <c r="S150" s="3"/>
       <c r="T150" s="3"/>
       <c r="U150" s="3"/>
       <c r="V150" s="3"/>
@@ -12312,16 +12320,14 @@
       <c r="AA150" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB150" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB150" s="3"/>
     </row>
     <row r="151" spans="1:28">
       <c r="A151" s="7">
         <v>149</v>
       </c>
       <c r="B151" s="7">
-        <v>2026060049</v>
+        <v>2026060048</v>
       </c>
       <c r="C151" s="7">
         <v>1</v>
@@ -12342,10 +12348,10 @@
         <v>106</v>
       </c>
       <c r="I151" s="7" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="J151" s="7" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="K151" s="7" t="s">
         <v>36</v>
@@ -12354,20 +12360,22 @@
         <v>377</v>
       </c>
       <c r="M151" s="8" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="N151" s="8" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="O151" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P151" s="7"/>
       <c r="Q151" s="7"/>
       <c r="R151" s="7">
         <v>5766</v>
       </c>
-      <c r="S151" s="7"/>
+      <c r="S151" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T151" s="7"/>
       <c r="U151" s="7"/>
       <c r="V151" s="7"/>
@@ -12380,14 +12388,16 @@
       <c r="AA151" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB151" s="7"/>
+      <c r="AB151" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="152" spans="1:28">
       <c r="A152" s="3">
         <v>150</v>
       </c>
       <c r="B152" s="3">
-        <v>2026061105</v>
+        <v>2026060049</v>
       </c>
       <c r="C152" s="3">
         <v>1</v>
@@ -12399,7 +12409,7 @@
         <v>345</v>
       </c>
       <c r="F152" s="3" t="s">
-        <v>42</v>
+        <v>209</v>
       </c>
       <c r="G152" s="3" t="s">
         <v>137</v>
@@ -12408,32 +12418,32 @@
         <v>106</v>
       </c>
       <c r="I152" s="3" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="J152" s="3" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="K152" s="3" t="s">
         <v>36</v>
       </c>
       <c r="L152" s="6" t="s">
+        <v>377</v>
+      </c>
+      <c r="M152" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="N152" s="6" t="s">
         <v>440</v>
       </c>
-      <c r="M152" s="6" t="s">
-        <v>441</v>
-      </c>
-      <c r="N152" s="6"/>
       <c r="O152" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P152" s="3"/>
       <c r="Q152" s="3"/>
       <c r="R152" s="3">
-        <v>167548</v>
-      </c>
-      <c r="S152" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>5766</v>
+      </c>
+      <c r="S152" s="3"/>
       <c r="T152" s="3"/>
       <c r="U152" s="3"/>
       <c r="V152" s="3"/>
@@ -12446,16 +12456,14 @@
       <c r="AA152" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB152" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB152" s="3"/>
     </row>
     <row r="153" spans="1:28">
       <c r="A153" s="7">
         <v>151</v>
       </c>
       <c r="B153" s="7">
-        <v>2026061106</v>
+        <v>2026061105</v>
       </c>
       <c r="C153" s="7">
         <v>1</v>
@@ -12476,30 +12484,32 @@
         <v>106</v>
       </c>
       <c r="I153" s="7" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="J153" s="7" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="K153" s="7" t="s">
         <v>36</v>
       </c>
       <c r="L153" s="8" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="M153" s="8" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="N153" s="8"/>
       <c r="O153" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P153" s="7"/>
       <c r="Q153" s="7"/>
       <c r="R153" s="7">
         <v>167548</v>
       </c>
-      <c r="S153" s="7"/>
+      <c r="S153" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T153" s="7"/>
       <c r="U153" s="7"/>
       <c r="V153" s="7"/>
@@ -12512,14 +12522,16 @@
       <c r="AA153" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB153" s="7"/>
+      <c r="AB153" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="154" spans="1:28">
       <c r="A154" s="3">
         <v>152</v>
       </c>
       <c r="B154" s="3">
-        <v>2026060819</v>
+        <v>2026061106</v>
       </c>
       <c r="C154" s="3">
         <v>1</v>
@@ -12531,45 +12543,39 @@
         <v>345</v>
       </c>
       <c r="F154" s="3" t="s">
-        <v>113</v>
+        <v>42</v>
       </c>
       <c r="G154" s="3" t="s">
-        <v>303</v>
+        <v>137</v>
       </c>
       <c r="H154" s="3" t="s">
-        <v>315</v>
+        <v>106</v>
       </c>
       <c r="I154" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="J154" s="3" t="s">
-        <v>133</v>
+        <v>428</v>
       </c>
       <c r="K154" s="3" t="s">
         <v>36</v>
       </c>
       <c r="L154" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="M154" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="M154" s="6" t="s">
-        <v>444</v>
-      </c>
-      <c r="N154" s="6" t="s">
-        <v>358</v>
-      </c>
+      <c r="N154" s="6"/>
       <c r="O154" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P154" s="3"/>
-      <c r="Q154" s="3">
-        <v>35761</v>
-      </c>
+      <c r="Q154" s="3"/>
       <c r="R154" s="3">
-        <v>68540</v>
-      </c>
-      <c r="S154" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>167548</v>
+      </c>
+      <c r="S154" s="3"/>
       <c r="T154" s="3"/>
       <c r="U154" s="3"/>
       <c r="V154" s="3"/>
@@ -12579,7 +12585,9 @@
       <c r="Z154" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="AA154" s="3"/>
+      <c r="AA154" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="AB154" s="3"/>
     </row>
     <row r="155" spans="1:28">
@@ -12587,7 +12595,7 @@
         <v>153</v>
       </c>
       <c r="B155" s="7">
-        <v>2026060820</v>
+        <v>2026060819</v>
       </c>
       <c r="C155" s="7">
         <v>1</v>
@@ -12608,7 +12616,7 @@
         <v>315</v>
       </c>
       <c r="I155" s="7" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="J155" s="7" t="s">
         <v>133</v>
@@ -12617,16 +12625,16 @@
         <v>36</v>
       </c>
       <c r="L155" s="8" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="M155" s="8" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="N155" s="8" t="s">
         <v>358</v>
       </c>
       <c r="O155" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P155" s="7"/>
       <c r="Q155" s="7">
@@ -12635,7 +12643,9 @@
       <c r="R155" s="7">
         <v>68540</v>
       </c>
-      <c r="S155" s="7"/>
+      <c r="S155" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T155" s="7"/>
       <c r="U155" s="7"/>
       <c r="V155" s="7"/>
@@ -12645,9 +12655,7 @@
       <c r="Z155" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="AA155" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA155" s="7"/>
       <c r="AB155" s="7"/>
     </row>
     <row r="156" spans="1:28">
@@ -12655,7 +12663,7 @@
         <v>154</v>
       </c>
       <c r="B156" s="3">
-        <v>2026060922</v>
+        <v>2026060820</v>
       </c>
       <c r="C156" s="3">
         <v>1</v>
@@ -12667,7 +12675,7 @@
         <v>345</v>
       </c>
       <c r="F156" s="3" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="G156" s="3" t="s">
         <v>303</v>
@@ -12676,7 +12684,7 @@
         <v>315</v>
       </c>
       <c r="I156" s="3" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="J156" s="3" t="s">
         <v>133</v>
@@ -12685,16 +12693,16 @@
         <v>36</v>
       </c>
       <c r="L156" s="6" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="M156" s="6" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="N156" s="6" t="s">
         <v>358</v>
       </c>
       <c r="O156" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P156" s="3"/>
       <c r="Q156" s="3">
@@ -12707,27 +12715,23 @@
       <c r="T156" s="3"/>
       <c r="U156" s="3"/>
       <c r="V156" s="3"/>
-      <c r="W156" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="W156" s="3"/>
       <c r="X156" s="3"/>
       <c r="Y156" s="3"/>
       <c r="Z156" s="6" t="s">
-        <v>366</v>
+        <v>349</v>
       </c>
       <c r="AA156" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB156" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB156" s="3"/>
     </row>
     <row r="157" spans="1:28">
       <c r="A157" s="7">
         <v>155</v>
       </c>
       <c r="B157" s="7">
-        <v>2026060527</v>
+        <v>2026060922</v>
       </c>
       <c r="C157" s="7">
         <v>1</v>
@@ -12739,49 +12743,53 @@
         <v>345</v>
       </c>
       <c r="F157" s="7" t="s">
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="G157" s="7" t="s">
-        <v>210</v>
+        <v>303</v>
       </c>
       <c r="H157" s="7" t="s">
-        <v>75</v>
+        <v>315</v>
       </c>
       <c r="I157" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="J157" s="7" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="K157" s="7" t="s">
         <v>36</v>
       </c>
       <c r="L157" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="M157" s="8" t="s">
         <v>446</v>
       </c>
-      <c r="M157" s="8" t="s">
-        <v>447</v>
-      </c>
       <c r="N157" s="8" t="s">
-        <v>448</v>
+        <v>358</v>
       </c>
       <c r="O157" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P157" s="7"/>
-      <c r="Q157" s="7"/>
+      <c r="Q157" s="7">
+        <v>35761</v>
+      </c>
       <c r="R157" s="7">
-        <v>33686</v>
+        <v>68540</v>
       </c>
       <c r="S157" s="7"/>
       <c r="T157" s="7"/>
       <c r="U157" s="7"/>
       <c r="V157" s="7"/>
-      <c r="W157" s="7"/>
+      <c r="W157" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="X157" s="7"/>
       <c r="Y157" s="7"/>
       <c r="Z157" s="8" t="s">
-        <v>349</v>
+        <v>366</v>
       </c>
       <c r="AA157" s="7" t="s">
         <v>40</v>
@@ -12816,7 +12824,7 @@
         <v>75</v>
       </c>
       <c r="I158" s="3" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="J158" s="3" t="s">
         <v>140</v>
@@ -12825,13 +12833,13 @@
         <v>36</v>
       </c>
       <c r="L158" s="6" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="M158" s="6" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="N158" s="6" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="O158" s="3" t="s">
         <v>39</v>
@@ -12861,7 +12869,7 @@
         <v>157</v>
       </c>
       <c r="B159" s="7">
-        <v>2026060408</v>
+        <v>2026060527</v>
       </c>
       <c r="C159" s="7">
         <v>1</v>
@@ -12876,13 +12884,13 @@
         <v>49</v>
       </c>
       <c r="G159" s="7" t="s">
-        <v>43</v>
+        <v>210</v>
       </c>
       <c r="H159" s="7" t="s">
-        <v>257</v>
+        <v>75</v>
       </c>
       <c r="I159" s="7" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="J159" s="7" t="s">
         <v>140</v>
@@ -12891,25 +12899,23 @@
         <v>36</v>
       </c>
       <c r="L159" s="8" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="M159" s="8" t="s">
+        <v>449</v>
+      </c>
+      <c r="N159" s="8" t="s">
         <v>450</v>
       </c>
-      <c r="N159" s="8" t="s">
-        <v>451</v>
-      </c>
       <c r="O159" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P159" s="7"/>
       <c r="Q159" s="7"/>
       <c r="R159" s="7">
-        <v>19776</v>
-      </c>
-      <c r="S159" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>33686</v>
+      </c>
+      <c r="S159" s="7"/>
       <c r="T159" s="7"/>
       <c r="U159" s="7"/>
       <c r="V159" s="7"/>
@@ -12919,7 +12925,9 @@
       <c r="Z159" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="AA159" s="7"/>
+      <c r="AA159" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="AB159" s="7"/>
     </row>
     <row r="160" spans="1:28">
@@ -12927,7 +12935,7 @@
         <v>158</v>
       </c>
       <c r="B160" s="3">
-        <v>2026060409</v>
+        <v>2026060408</v>
       </c>
       <c r="C160" s="3">
         <v>1</v>
@@ -12948,7 +12956,7 @@
         <v>257</v>
       </c>
       <c r="I160" s="3" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="J160" s="3" t="s">
         <v>140</v>
@@ -12957,23 +12965,25 @@
         <v>36</v>
       </c>
       <c r="L160" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M160" s="6" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="N160" s="6" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="O160" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P160" s="3"/>
       <c r="Q160" s="3"/>
       <c r="R160" s="3">
         <v>19776</v>
       </c>
-      <c r="S160" s="3"/>
+      <c r="S160" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T160" s="3"/>
       <c r="U160" s="3"/>
       <c r="V160" s="3"/>
@@ -12983,9 +12993,7 @@
       <c r="Z160" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="AA160" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA160" s="3"/>
       <c r="AB160" s="3"/>
     </row>
     <row r="161" spans="1:28">
@@ -12993,7 +13001,7 @@
         <v>159</v>
       </c>
       <c r="B161" s="7">
-        <v>2026060389</v>
+        <v>2026060409</v>
       </c>
       <c r="C161" s="7">
         <v>1</v>
@@ -13008,13 +13016,13 @@
         <v>49</v>
       </c>
       <c r="G161" s="7" t="s">
-        <v>137</v>
+        <v>43</v>
       </c>
       <c r="H161" s="7" t="s">
-        <v>106</v>
+        <v>257</v>
       </c>
       <c r="I161" s="7" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="J161" s="7" t="s">
         <v>140</v>
@@ -13023,25 +13031,23 @@
         <v>36</v>
       </c>
       <c r="L161" s="8" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M161" s="8" t="s">
+        <v>452</v>
+      </c>
+      <c r="N161" s="8" t="s">
         <v>453</v>
       </c>
-      <c r="N161" s="8" t="s">
-        <v>454</v>
-      </c>
       <c r="O161" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P161" s="7"/>
       <c r="Q161" s="7"/>
       <c r="R161" s="7">
-        <v>92779</v>
-      </c>
-      <c r="S161" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>19776</v>
+      </c>
+      <c r="S161" s="7"/>
       <c r="T161" s="7"/>
       <c r="U161" s="7"/>
       <c r="V161" s="7"/>
@@ -13051,7 +13057,9 @@
       <c r="Z161" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="AA161" s="7"/>
+      <c r="AA161" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="AB161" s="7"/>
     </row>
     <row r="162" spans="1:28">
@@ -13059,7 +13067,7 @@
         <v>160</v>
       </c>
       <c r="B162" s="3">
-        <v>2026060390</v>
+        <v>2026060389</v>
       </c>
       <c r="C162" s="3">
         <v>1</v>
@@ -13080,7 +13088,7 @@
         <v>106</v>
       </c>
       <c r="I162" s="3" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="J162" s="3" t="s">
         <v>140</v>
@@ -13089,23 +13097,25 @@
         <v>36</v>
       </c>
       <c r="L162" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M162" s="6" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="N162" s="6" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="O162" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P162" s="3"/>
       <c r="Q162" s="3"/>
       <c r="R162" s="3">
         <v>92779</v>
       </c>
-      <c r="S162" s="3"/>
+      <c r="S162" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T162" s="3"/>
       <c r="U162" s="3"/>
       <c r="V162" s="3"/>
@@ -13115,9 +13125,7 @@
       <c r="Z162" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="AA162" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA162" s="3"/>
       <c r="AB162" s="3"/>
     </row>
     <row r="163" spans="1:28">
@@ -13125,7 +13133,7 @@
         <v>161</v>
       </c>
       <c r="B163" s="7">
-        <v>2026060853</v>
+        <v>2026060390</v>
       </c>
       <c r="C163" s="7">
         <v>1</v>
@@ -13137,16 +13145,16 @@
         <v>345</v>
       </c>
       <c r="F163" s="7" t="s">
-        <v>113</v>
+        <v>49</v>
       </c>
       <c r="G163" s="7" t="s">
-        <v>105</v>
+        <v>137</v>
       </c>
       <c r="H163" s="7" t="s">
-        <v>234</v>
+        <v>106</v>
       </c>
       <c r="I163" s="7" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="J163" s="7" t="s">
         <v>140</v>
@@ -13155,16 +13163,16 @@
         <v>36</v>
       </c>
       <c r="L163" s="8" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M163" s="8" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="N163" s="8" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="O163" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P163" s="7"/>
       <c r="Q163" s="7"/>
@@ -13177,25 +13185,21 @@
       <c r="V163" s="7"/>
       <c r="W163" s="7"/>
       <c r="X163" s="7"/>
-      <c r="Y163" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="Y163" s="7"/>
       <c r="Z163" s="8" t="s">
-        <v>455</v>
+        <v>349</v>
       </c>
       <c r="AA163" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB163" s="7">
-        <v>1</v>
-      </c>
+      <c r="AB163" s="7"/>
     </row>
     <row r="164" spans="1:28">
       <c r="A164" s="3">
         <v>162</v>
       </c>
       <c r="B164" s="3">
-        <v>2026060383</v>
+        <v>2026060853</v>
       </c>
       <c r="C164" s="3">
         <v>1</v>
@@ -13207,16 +13211,16 @@
         <v>345</v>
       </c>
       <c r="F164" s="3" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="G164" s="3" t="s">
-        <v>354</v>
+        <v>105</v>
       </c>
       <c r="H164" s="3" t="s">
-        <v>202</v>
+        <v>234</v>
       </c>
       <c r="I164" s="3" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="J164" s="3" t="s">
         <v>140</v>
@@ -13225,13 +13229,13 @@
         <v>36</v>
       </c>
       <c r="L164" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M164" s="6" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="N164" s="6" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="O164" s="3" t="s">
         <v>39</v>
@@ -13239,29 +13243,33 @@
       <c r="P164" s="3"/>
       <c r="Q164" s="3"/>
       <c r="R164" s="3">
-        <v>207716</v>
-      </c>
-      <c r="S164" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>92779</v>
+      </c>
+      <c r="S164" s="3"/>
       <c r="T164" s="3"/>
       <c r="U164" s="3"/>
       <c r="V164" s="3"/>
       <c r="W164" s="3"/>
       <c r="X164" s="3"/>
-      <c r="Y164" s="3"/>
+      <c r="Y164" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="Z164" s="6" t="s">
-        <v>349</v>
-      </c>
-      <c r="AA164" s="3"/>
-      <c r="AB164" s="3"/>
+        <v>457</v>
+      </c>
+      <c r="AA164" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB164" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="165" spans="1:28">
       <c r="A165" s="7">
         <v>163</v>
       </c>
       <c r="B165" s="7">
-        <v>2026060384</v>
+        <v>2026060383</v>
       </c>
       <c r="C165" s="7">
         <v>1</v>
@@ -13282,7 +13290,7 @@
         <v>202</v>
       </c>
       <c r="I165" s="7" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="J165" s="7" t="s">
         <v>140</v>
@@ -13291,23 +13299,25 @@
         <v>36</v>
       </c>
       <c r="L165" s="8" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M165" s="8" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="N165" s="8" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="O165" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P165" s="7"/>
       <c r="Q165" s="7"/>
       <c r="R165" s="7">
         <v>207716</v>
       </c>
-      <c r="S165" s="7"/>
+      <c r="S165" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T165" s="7"/>
       <c r="U165" s="7"/>
       <c r="V165" s="7"/>
@@ -13317,9 +13327,7 @@
       <c r="Z165" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="AA165" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA165" s="7"/>
       <c r="AB165" s="7"/>
     </row>
     <row r="166" spans="1:28">
@@ -13327,7 +13335,7 @@
         <v>164</v>
       </c>
       <c r="B166" s="3">
-        <v>2026060569</v>
+        <v>2026060384</v>
       </c>
       <c r="C166" s="3">
         <v>1</v>
@@ -13342,13 +13350,13 @@
         <v>49</v>
       </c>
       <c r="G166" s="3" t="s">
-        <v>303</v>
+        <v>354</v>
       </c>
       <c r="H166" s="3" t="s">
-        <v>315</v>
+        <v>202</v>
       </c>
       <c r="I166" s="3" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="J166" s="3" t="s">
         <v>140</v>
@@ -13357,16 +13365,16 @@
         <v>36</v>
       </c>
       <c r="L166" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M166" s="6" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="N166" s="6" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="O166" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P166" s="3"/>
       <c r="Q166" s="3"/>
@@ -13375,29 +13383,25 @@
       </c>
       <c r="S166" s="3"/>
       <c r="T166" s="3"/>
-      <c r="U166" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="U166" s="3"/>
       <c r="V166" s="3"/>
       <c r="W166" s="3"/>
       <c r="X166" s="3"/>
       <c r="Y166" s="3"/>
       <c r="Z166" s="6" t="s">
-        <v>403</v>
+        <v>349</v>
       </c>
       <c r="AA166" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB166" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB166" s="3"/>
     </row>
     <row r="167" spans="1:28">
       <c r="A167" s="7">
         <v>165</v>
       </c>
       <c r="B167" s="7">
-        <v>2026060387</v>
+        <v>2026060569</v>
       </c>
       <c r="C167" s="7">
         <v>1</v>
@@ -13412,13 +13416,13 @@
         <v>49</v>
       </c>
       <c r="G167" s="7" t="s">
-        <v>50</v>
+        <v>303</v>
       </c>
       <c r="H167" s="7" t="s">
-        <v>137</v>
+        <v>315</v>
       </c>
       <c r="I167" s="7" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="J167" s="7" t="s">
         <v>140</v>
@@ -13427,13 +13431,13 @@
         <v>36</v>
       </c>
       <c r="L167" s="8" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M167" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="N167" s="8" t="s">
         <v>460</v>
-      </c>
-      <c r="N167" s="8" t="s">
-        <v>461</v>
       </c>
       <c r="O167" s="7" t="s">
         <v>39</v>
@@ -13441,29 +13445,33 @@
       <c r="P167" s="7"/>
       <c r="Q167" s="7"/>
       <c r="R167" s="7">
-        <v>152071</v>
-      </c>
-      <c r="S167" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>207716</v>
+      </c>
+      <c r="S167" s="7"/>
       <c r="T167" s="7"/>
-      <c r="U167" s="7"/>
+      <c r="U167" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="V167" s="7"/>
       <c r="W167" s="7"/>
       <c r="X167" s="7"/>
       <c r="Y167" s="7"/>
       <c r="Z167" s="8" t="s">
-        <v>349</v>
-      </c>
-      <c r="AA167" s="7"/>
-      <c r="AB167" s="7"/>
+        <v>403</v>
+      </c>
+      <c r="AA167" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB167" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="168" spans="1:28">
       <c r="A168" s="3">
         <v>166</v>
       </c>
       <c r="B168" s="3">
-        <v>2026060388</v>
+        <v>2026060387</v>
       </c>
       <c r="C168" s="3">
         <v>1</v>
@@ -13484,7 +13492,7 @@
         <v>137</v>
       </c>
       <c r="I168" s="3" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="J168" s="3" t="s">
         <v>140</v>
@@ -13493,23 +13501,25 @@
         <v>36</v>
       </c>
       <c r="L168" s="6" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M168" s="6" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="N168" s="6" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="O168" s="3" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P168" s="3"/>
       <c r="Q168" s="3"/>
       <c r="R168" s="3">
         <v>152071</v>
       </c>
-      <c r="S168" s="3"/>
+      <c r="S168" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T168" s="3"/>
       <c r="U168" s="3"/>
       <c r="V168" s="3"/>
@@ -13519,9 +13529,7 @@
       <c r="Z168" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="AA168" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA168" s="3"/>
       <c r="AB168" s="3"/>
     </row>
     <row r="169" spans="1:28">
@@ -13529,7 +13537,7 @@
         <v>167</v>
       </c>
       <c r="B169" s="7">
-        <v>2026060570</v>
+        <v>2026060388</v>
       </c>
       <c r="C169" s="7">
         <v>1</v>
@@ -13544,13 +13552,13 @@
         <v>49</v>
       </c>
       <c r="G169" s="7" t="s">
-        <v>315</v>
+        <v>50</v>
       </c>
       <c r="H169" s="7" t="s">
-        <v>164</v>
+        <v>137</v>
       </c>
       <c r="I169" s="7" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="J169" s="7" t="s">
         <v>140</v>
@@ -13559,16 +13567,16 @@
         <v>36</v>
       </c>
       <c r="L169" s="8" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="M169" s="8" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="N169" s="8" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="O169" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P169" s="7"/>
       <c r="Q169" s="7"/>
@@ -13577,29 +13585,25 @@
       </c>
       <c r="S169" s="7"/>
       <c r="T169" s="7"/>
-      <c r="U169" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="U169" s="7"/>
       <c r="V169" s="7"/>
       <c r="W169" s="7"/>
       <c r="X169" s="7"/>
       <c r="Y169" s="7"/>
       <c r="Z169" s="8" t="s">
-        <v>403</v>
+        <v>349</v>
       </c>
       <c r="AA169" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB169" s="7">
-        <v>1</v>
-      </c>
+      <c r="AB169" s="7"/>
     </row>
     <row r="170" spans="1:28">
       <c r="A170" s="3">
         <v>168</v>
       </c>
       <c r="B170" s="3">
-        <v>2026061402</v>
+        <v>2026060570</v>
       </c>
       <c r="C170" s="3">
         <v>1</v>
@@ -13611,31 +13615,31 @@
         <v>345</v>
       </c>
       <c r="F170" s="3" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="G170" s="3" t="s">
-        <v>359</v>
+        <v>315</v>
       </c>
       <c r="H170" s="3" t="s">
-        <v>354</v>
+        <v>164</v>
       </c>
       <c r="I170" s="3" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="J170" s="3" t="s">
-        <v>463</v>
+        <v>140</v>
       </c>
       <c r="K170" s="3" t="s">
         <v>36</v>
       </c>
       <c r="L170" s="6" t="s">
-        <v>464</v>
+        <v>429</v>
       </c>
       <c r="M170" s="6" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="N170" s="6" t="s">
-        <v>383</v>
+        <v>463</v>
       </c>
       <c r="O170" s="3" t="s">
         <v>39</v>
@@ -13643,29 +13647,33 @@
       <c r="P170" s="3"/>
       <c r="Q170" s="3"/>
       <c r="R170" s="3">
-        <v>6530</v>
-      </c>
-      <c r="S170" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>152071</v>
+      </c>
+      <c r="S170" s="3"/>
       <c r="T170" s="3"/>
-      <c r="U170" s="3"/>
+      <c r="U170" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="V170" s="3"/>
       <c r="W170" s="3"/>
       <c r="X170" s="3"/>
       <c r="Y170" s="3"/>
       <c r="Z170" s="6" t="s">
-        <v>349</v>
-      </c>
-      <c r="AA170" s="3"/>
-      <c r="AB170" s="3"/>
+        <v>403</v>
+      </c>
+      <c r="AA170" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB170" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="171" spans="1:28">
       <c r="A171" s="7">
         <v>169</v>
       </c>
       <c r="B171" s="7">
-        <v>2026061403</v>
+        <v>2026061402</v>
       </c>
       <c r="C171" s="7">
         <v>1</v>
@@ -13686,32 +13694,34 @@
         <v>354</v>
       </c>
       <c r="I171" s="7" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="J171" s="7" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="K171" s="7" t="s">
         <v>36</v>
       </c>
       <c r="L171" s="8" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="M171" s="8" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="N171" s="8" t="s">
         <v>383</v>
       </c>
       <c r="O171" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P171" s="7"/>
       <c r="Q171" s="7"/>
       <c r="R171" s="7">
         <v>6530</v>
       </c>
-      <c r="S171" s="7"/>
+      <c r="S171" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T171" s="7"/>
       <c r="U171" s="7"/>
       <c r="V171" s="7"/>
@@ -13721,9 +13731,7 @@
       <c r="Z171" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="AA171" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA171" s="7"/>
       <c r="AB171" s="7"/>
     </row>
     <row r="172" spans="1:28">
@@ -13731,7 +13739,7 @@
         <v>170</v>
       </c>
       <c r="B172" s="3">
-        <v>2026060081</v>
+        <v>2026061403</v>
       </c>
       <c r="C172" s="3">
         <v>1</v>
@@ -13743,43 +13751,41 @@
         <v>345</v>
       </c>
       <c r="F172" s="3" t="s">
-        <v>209</v>
+        <v>31</v>
       </c>
       <c r="G172" s="3" t="s">
-        <v>315</v>
+        <v>359</v>
       </c>
       <c r="H172" s="3" t="s">
-        <v>164</v>
+        <v>354</v>
       </c>
       <c r="I172" s="3" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="J172" s="3" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="K172" s="3" t="s">
         <v>36</v>
       </c>
       <c r="L172" s="6" t="s">
-        <v>400</v>
+        <v>466</v>
       </c>
       <c r="M172" s="6" t="s">
         <v>467</v>
       </c>
       <c r="N172" s="6" t="s">
-        <v>468</v>
+        <v>383</v>
       </c>
       <c r="O172" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P172" s="3"/>
       <c r="Q172" s="3"/>
       <c r="R172" s="3">
-        <v>48</v>
-      </c>
-      <c r="S172" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>6530</v>
+      </c>
+      <c r="S172" s="3"/>
       <c r="T172" s="3"/>
       <c r="U172" s="3"/>
       <c r="V172" s="3"/>
@@ -13789,7 +13795,9 @@
       <c r="Z172" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="AA172" s="3"/>
+      <c r="AA172" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="AB172" s="3"/>
     </row>
     <row r="173" spans="1:28">
@@ -13797,7 +13805,7 @@
         <v>171</v>
       </c>
       <c r="B173" s="7">
-        <v>2026060082</v>
+        <v>2026060081</v>
       </c>
       <c r="C173" s="7">
         <v>1</v>
@@ -13818,10 +13826,10 @@
         <v>164</v>
       </c>
       <c r="I173" s="7" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="J173" s="7" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="K173" s="7" t="s">
         <v>36</v>
@@ -13830,20 +13838,22 @@
         <v>400</v>
       </c>
       <c r="M173" s="8" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="N173" s="8" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="O173" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P173" s="7"/>
       <c r="Q173" s="7"/>
       <c r="R173" s="7">
         <v>48</v>
       </c>
-      <c r="S173" s="7"/>
+      <c r="S173" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T173" s="7"/>
       <c r="U173" s="7"/>
       <c r="V173" s="7"/>
@@ -13853,9 +13863,7 @@
       <c r="Z173" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="AA173" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA173" s="7"/>
       <c r="AB173" s="7"/>
     </row>
     <row r="174" spans="1:28">
@@ -13863,7 +13871,7 @@
         <v>172</v>
       </c>
       <c r="B174" s="3">
-        <v>2026061407</v>
+        <v>2026060082</v>
       </c>
       <c r="C174" s="3">
         <v>1</v>
@@ -13875,43 +13883,41 @@
         <v>345</v>
       </c>
       <c r="F174" s="3" t="s">
-        <v>31</v>
+        <v>209</v>
       </c>
       <c r="G174" s="3" t="s">
-        <v>202</v>
+        <v>315</v>
       </c>
       <c r="H174" s="3" t="s">
-        <v>50</v>
+        <v>164</v>
       </c>
       <c r="I174" s="3" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="J174" s="3" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="K174" s="3" t="s">
         <v>36</v>
       </c>
       <c r="L174" s="6" t="s">
-        <v>373</v>
+        <v>400</v>
       </c>
       <c r="M174" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="N174" s="6" t="s">
         <v>470</v>
       </c>
-      <c r="N174" s="6" t="s">
-        <v>432</v>
-      </c>
       <c r="O174" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P174" s="3"/>
       <c r="Q174" s="3"/>
       <c r="R174" s="3">
-        <v>478</v>
-      </c>
-      <c r="S174" s="3" t="s">
-        <v>40</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="S174" s="3"/>
       <c r="T174" s="3"/>
       <c r="U174" s="3"/>
       <c r="V174" s="3"/>
@@ -13921,7 +13927,9 @@
       <c r="Z174" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="AA174" s="3"/>
+      <c r="AA174" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="AB174" s="3"/>
     </row>
     <row r="175" spans="1:28">
@@ -13929,7 +13937,7 @@
         <v>173</v>
       </c>
       <c r="B175" s="7">
-        <v>2026061408</v>
+        <v>2026061407</v>
       </c>
       <c r="C175" s="7">
         <v>1</v>
@@ -13950,10 +13958,10 @@
         <v>50</v>
       </c>
       <c r="I175" s="7" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="J175" s="7" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="K175" s="7" t="s">
         <v>36</v>
@@ -13962,20 +13970,22 @@
         <v>373</v>
       </c>
       <c r="M175" s="8" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="N175" s="8" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="O175" s="7" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="P175" s="7"/>
       <c r="Q175" s="7"/>
       <c r="R175" s="7">
         <v>478</v>
       </c>
-      <c r="S175" s="7"/>
+      <c r="S175" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T175" s="7"/>
       <c r="U175" s="7"/>
       <c r="V175" s="7"/>
@@ -13985,9 +13995,7 @@
       <c r="Z175" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="AA175" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="AA175" s="7"/>
       <c r="AB175" s="7"/>
     </row>
     <row r="176" spans="1:28">
@@ -13995,7 +14003,7 @@
         <v>174</v>
       </c>
       <c r="B176" s="3">
-        <v>2026060145</v>
+        <v>2026061408</v>
       </c>
       <c r="C176" s="3">
         <v>1</v>
@@ -14007,65 +14015,61 @@
         <v>345</v>
       </c>
       <c r="F176" s="3" t="s">
-        <v>209</v>
+        <v>31</v>
       </c>
       <c r="G176" s="3" t="s">
-        <v>143</v>
+        <v>202</v>
       </c>
       <c r="H176" s="3" t="s">
-        <v>165</v>
+        <v>50</v>
       </c>
       <c r="I176" s="3" t="s">
         <v>471</v>
       </c>
       <c r="J176" s="3" t="s">
-        <v>265</v>
+        <v>465</v>
       </c>
       <c r="K176" s="3" t="s">
         <v>36</v>
       </c>
       <c r="L176" s="6" t="s">
-        <v>400</v>
+        <v>373</v>
       </c>
       <c r="M176" s="6" t="s">
         <v>472</v>
       </c>
       <c r="N176" s="6" t="s">
-        <v>473</v>
+        <v>434</v>
       </c>
       <c r="O176" s="3" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="P176" s="3"/>
       <c r="Q176" s="3"/>
       <c r="R176" s="3">
-        <v>38244</v>
+        <v>478</v>
       </c>
       <c r="S176" s="3"/>
       <c r="T176" s="3"/>
-      <c r="U176" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="U176" s="3"/>
       <c r="V176" s="3"/>
       <c r="W176" s="3"/>
       <c r="X176" s="3"/>
       <c r="Y176" s="3"/>
       <c r="Z176" s="6" t="s">
-        <v>403</v>
+        <v>349</v>
       </c>
       <c r="AA176" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB176" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB176" s="3"/>
     </row>
     <row r="177" spans="1:28">
       <c r="A177" s="7">
         <v>175</v>
       </c>
       <c r="B177" s="7">
-        <v>2026060144</v>
+        <v>2026060145</v>
       </c>
       <c r="C177" s="7">
         <v>1</v>
@@ -14080,13 +14084,13 @@
         <v>209</v>
       </c>
       <c r="G177" s="7" t="s">
-        <v>210</v>
+        <v>143</v>
       </c>
       <c r="H177" s="7" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="I177" s="7" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="J177" s="7" t="s">
         <v>265</v>
@@ -14098,7 +14102,7 @@
         <v>400</v>
       </c>
       <c r="M177" s="8" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="N177" s="8" t="s">
         <v>475</v>
@@ -14109,7 +14113,7 @@
       <c r="P177" s="7"/>
       <c r="Q177" s="7"/>
       <c r="R177" s="7">
-        <v>386259</v>
+        <v>38244</v>
       </c>
       <c r="S177" s="7"/>
       <c r="T177" s="7"/>
@@ -14135,7 +14139,7 @@
         <v>176</v>
       </c>
       <c r="B178" s="3">
-        <v>2026060143</v>
+        <v>2026060144</v>
       </c>
       <c r="C178" s="3">
         <v>1</v>
@@ -14150,10 +14154,10 @@
         <v>209</v>
       </c>
       <c r="G178" s="3" t="s">
-        <v>291</v>
+        <v>210</v>
       </c>
       <c r="H178" s="3" t="s">
-        <v>210</v>
+        <v>143</v>
       </c>
       <c r="I178" s="3" t="s">
         <v>476</v>
@@ -14168,7 +14172,7 @@
         <v>400</v>
       </c>
       <c r="M178" s="6" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="N178" s="6" t="s">
         <v>477</v>
@@ -14179,7 +14183,7 @@
       <c r="P178" s="3"/>
       <c r="Q178" s="3"/>
       <c r="R178" s="3">
-        <v>381383</v>
+        <v>386259</v>
       </c>
       <c r="S178" s="3"/>
       <c r="T178" s="3"/>
@@ -14205,7 +14209,7 @@
         <v>177</v>
       </c>
       <c r="B179" s="7">
-        <v>2026060142</v>
+        <v>2026060143</v>
       </c>
       <c r="C179" s="7">
         <v>1</v>
@@ -14220,10 +14224,10 @@
         <v>209</v>
       </c>
       <c r="G179" s="7" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H179" s="7" t="s">
-        <v>291</v>
+        <v>210</v>
       </c>
       <c r="I179" s="7" t="s">
         <v>478</v>
@@ -14238,7 +14242,7 @@
         <v>400</v>
       </c>
       <c r="M179" s="8" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="N179" s="8" t="s">
         <v>479</v>
@@ -14249,7 +14253,7 @@
       <c r="P179" s="7"/>
       <c r="Q179" s="7"/>
       <c r="R179" s="7">
-        <v>31873</v>
+        <v>381383</v>
       </c>
       <c r="S179" s="7"/>
       <c r="T179" s="7"/>
@@ -14275,7 +14279,7 @@
         <v>178</v>
       </c>
       <c r="B180" s="3">
-        <v>2026060141</v>
+        <v>2026060142</v>
       </c>
       <c r="C180" s="3">
         <v>1</v>
@@ -14290,10 +14294,10 @@
         <v>209</v>
       </c>
       <c r="G180" s="3" t="s">
-        <v>225</v>
+        <v>290</v>
       </c>
       <c r="H180" s="3" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="I180" s="3" t="s">
         <v>480</v>
@@ -14308,7 +14312,7 @@
         <v>400</v>
       </c>
       <c r="M180" s="6" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="N180" s="6" t="s">
         <v>481</v>
@@ -14319,7 +14323,7 @@
       <c r="P180" s="3"/>
       <c r="Q180" s="3"/>
       <c r="R180" s="3">
-        <v>30842</v>
+        <v>31873</v>
       </c>
       <c r="S180" s="3"/>
       <c r="T180" s="3"/>
@@ -14345,7 +14349,7 @@
         <v>179</v>
       </c>
       <c r="B181" s="7">
-        <v>2026061273</v>
+        <v>2026060141</v>
       </c>
       <c r="C181" s="7">
         <v>1</v>
@@ -14357,27 +14361,31 @@
         <v>345</v>
       </c>
       <c r="F181" s="7" t="s">
-        <v>66</v>
+        <v>209</v>
       </c>
       <c r="G181" s="7" t="s">
-        <v>257</v>
+        <v>225</v>
       </c>
       <c r="H181" s="7" t="s">
-        <v>70</v>
+        <v>290</v>
       </c>
       <c r="I181" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="J181" s="7"/>
-      <c r="K181" s="7"/>
+      <c r="J181" s="7" t="s">
+        <v>265</v>
+      </c>
+      <c r="K181" s="7" t="s">
+        <v>36</v>
+      </c>
       <c r="L181" s="8" t="s">
-        <v>167</v>
+        <v>400</v>
       </c>
       <c r="M181" s="8" t="s">
+        <v>474</v>
+      </c>
+      <c r="N181" s="8" t="s">
         <v>483</v>
-      </c>
-      <c r="N181" s="8" t="s">
-        <v>484</v>
       </c>
       <c r="O181" s="7" t="s">
         <v>39</v>
@@ -14385,21 +14393,19 @@
       <c r="P181" s="7"/>
       <c r="Q181" s="7"/>
       <c r="R181" s="7">
-        <v>0</v>
-      </c>
-      <c r="S181" s="7" t="s">
-        <v>40</v>
-      </c>
+        <v>30842</v>
+      </c>
+      <c r="S181" s="7"/>
       <c r="T181" s="7"/>
-      <c r="U181" s="7"/>
+      <c r="U181" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="V181" s="7"/>
       <c r="W181" s="7"/>
       <c r="X181" s="7"/>
-      <c r="Y181" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="Y181" s="7"/>
       <c r="Z181" s="8" t="s">
-        <v>181</v>
+        <v>403</v>
       </c>
       <c r="AA181" s="7" t="s">
         <v>40</v>
@@ -14413,7 +14419,7 @@
         <v>180</v>
       </c>
       <c r="B182" s="3">
-        <v>2026060898</v>
+        <v>2026061273</v>
       </c>
       <c r="C182" s="3">
         <v>1</v>
@@ -14425,16 +14431,16 @@
         <v>345</v>
       </c>
       <c r="F182" s="3" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="G182" s="3" t="s">
-        <v>137</v>
+        <v>257</v>
       </c>
       <c r="H182" s="3" t="s">
-        <v>106</v>
+        <v>70</v>
       </c>
       <c r="I182" s="3" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="J182" s="3"/>
       <c r="K182" s="3"/>
@@ -14442,10 +14448,10 @@
         <v>167</v>
       </c>
       <c r="M182" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="N182" s="6" t="s">
         <v>486</v>
-      </c>
-      <c r="N182" s="6" t="s">
-        <v>487</v>
       </c>
       <c r="O182" s="3" t="s">
         <v>39</v>
@@ -14481,7 +14487,7 @@
         <v>181</v>
       </c>
       <c r="B183" s="7">
-        <v>2026060899</v>
+        <v>2026060898</v>
       </c>
       <c r="C183" s="7">
         <v>1</v>
@@ -14496,13 +14502,13 @@
         <v>87</v>
       </c>
       <c r="G183" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="H183" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="H183" s="7" t="s">
-        <v>43</v>
-      </c>
       <c r="I183" s="7" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J183" s="7"/>
       <c r="K183" s="7"/>
@@ -14510,10 +14516,10 @@
         <v>167</v>
       </c>
       <c r="M183" s="8" t="s">
+        <v>488</v>
+      </c>
+      <c r="N183" s="8" t="s">
         <v>489</v>
-      </c>
-      <c r="N183" s="8" t="s">
-        <v>490</v>
       </c>
       <c r="O183" s="7" t="s">
         <v>39</v>
@@ -14549,7 +14555,7 @@
         <v>182</v>
       </c>
       <c r="B184" s="3">
-        <v>2026060873</v>
+        <v>2026060899</v>
       </c>
       <c r="C184" s="3">
         <v>1</v>
@@ -14564,46 +14570,46 @@
         <v>87</v>
       </c>
       <c r="G184" s="3" t="s">
-        <v>315</v>
+        <v>106</v>
       </c>
       <c r="H184" s="3" t="s">
-        <v>164</v>
+        <v>43</v>
       </c>
       <c r="I184" s="3" t="s">
-        <v>491</v>
-      </c>
-      <c r="J184" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="K184" s="3" t="s">
-        <v>197</v>
-      </c>
+        <v>490</v>
+      </c>
+      <c r="J184" s="3"/>
+      <c r="K184" s="3"/>
       <c r="L184" s="6" t="s">
         <v>167</v>
       </c>
       <c r="M184" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="N184" s="6" t="s">
         <v>492</v>
       </c>
-      <c r="N184" s="6" t="s">
-        <v>493</v>
-      </c>
       <c r="O184" s="3" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="P184" s="3"/>
       <c r="Q184" s="3"/>
       <c r="R184" s="3">
         <v>0</v>
       </c>
-      <c r="S184" s="3"/>
+      <c r="S184" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T184" s="3"/>
       <c r="U184" s="3"/>
       <c r="V184" s="3"/>
       <c r="W184" s="3"/>
       <c r="X184" s="3"/>
-      <c r="Y184" s="3"/>
+      <c r="Y184" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="Z184" s="6" t="s">
-        <v>494</v>
+        <v>181</v>
       </c>
       <c r="AA184" s="3" t="s">
         <v>40</v>
@@ -14617,7 +14623,7 @@
         <v>183</v>
       </c>
       <c r="B185" s="7">
-        <v>2026061276</v>
+        <v>2026060873</v>
       </c>
       <c r="C185" s="7">
         <v>1</v>
@@ -14629,49 +14635,49 @@
         <v>345</v>
       </c>
       <c r="F185" s="7" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
       <c r="G185" s="7" t="s">
-        <v>70</v>
+        <v>315</v>
       </c>
       <c r="H185" s="7" t="s">
-        <v>303</v>
+        <v>164</v>
       </c>
       <c r="I185" s="7" t="s">
-        <v>495</v>
-      </c>
-      <c r="J185" s="7"/>
-      <c r="K185" s="7"/>
+        <v>493</v>
+      </c>
+      <c r="J185" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="K185" s="7" t="s">
+        <v>197</v>
+      </c>
       <c r="L185" s="8" t="s">
         <v>167</v>
       </c>
       <c r="M185" s="8" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="N185" s="8" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="O185" s="7" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="P185" s="7"/>
       <c r="Q185" s="7"/>
       <c r="R185" s="7">
         <v>0</v>
       </c>
-      <c r="S185" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S185" s="7"/>
       <c r="T185" s="7"/>
       <c r="U185" s="7"/>
       <c r="V185" s="7"/>
       <c r="W185" s="7"/>
       <c r="X185" s="7"/>
-      <c r="Y185" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="Y185" s="7"/>
       <c r="Z185" s="8" t="s">
-        <v>181</v>
+        <v>496</v>
       </c>
       <c r="AA185" s="7" t="s">
         <v>40</v>
@@ -14685,7 +14691,7 @@
         <v>184</v>
       </c>
       <c r="B186" s="3">
-        <v>2026061219</v>
+        <v>2026061276</v>
       </c>
       <c r="C186" s="3">
         <v>1</v>
@@ -14697,49 +14703,49 @@
         <v>345</v>
       </c>
       <c r="F186" s="3" t="s">
-        <v>298</v>
+        <v>66</v>
       </c>
       <c r="G186" s="3" t="s">
-        <v>210</v>
+        <v>70</v>
       </c>
       <c r="H186" s="3" t="s">
-        <v>234</v>
+        <v>303</v>
       </c>
       <c r="I186" s="3" t="s">
-        <v>498</v>
-      </c>
-      <c r="J186" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="K186" s="3" t="s">
-        <v>197</v>
-      </c>
+        <v>497</v>
+      </c>
+      <c r="J186" s="3"/>
+      <c r="K186" s="3"/>
       <c r="L186" s="6" t="s">
         <v>167</v>
       </c>
       <c r="M186" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="N186" s="6" t="s">
         <v>499</v>
       </c>
-      <c r="N186" s="6" t="s">
-        <v>500</v>
-      </c>
       <c r="O186" s="3" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="P186" s="3"/>
       <c r="Q186" s="3"/>
       <c r="R186" s="3">
         <v>0</v>
       </c>
-      <c r="S186" s="3"/>
+      <c r="S186" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T186" s="3"/>
       <c r="U186" s="3"/>
       <c r="V186" s="3"/>
       <c r="W186" s="3"/>
       <c r="X186" s="3"/>
-      <c r="Y186" s="3"/>
+      <c r="Y186" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="Z186" s="6" t="s">
-        <v>501</v>
+        <v>181</v>
       </c>
       <c r="AA186" s="3" t="s">
         <v>40</v>
@@ -14753,7 +14759,7 @@
         <v>185</v>
       </c>
       <c r="B187" s="7">
-        <v>2026061283</v>
+        <v>2026061219</v>
       </c>
       <c r="C187" s="7">
         <v>1</v>
@@ -14765,49 +14771,49 @@
         <v>345</v>
       </c>
       <c r="F187" s="7" t="s">
-        <v>66</v>
+        <v>298</v>
       </c>
       <c r="G187" s="7" t="s">
-        <v>303</v>
+        <v>210</v>
       </c>
       <c r="H187" s="7" t="s">
-        <v>315</v>
+        <v>234</v>
       </c>
       <c r="I187" s="7" t="s">
-        <v>498</v>
-      </c>
-      <c r="J187" s="7"/>
-      <c r="K187" s="7"/>
+        <v>500</v>
+      </c>
+      <c r="J187" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="K187" s="7" t="s">
+        <v>197</v>
+      </c>
       <c r="L187" s="8" t="s">
         <v>167</v>
       </c>
       <c r="M187" s="8" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="N187" s="8" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="O187" s="7" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="P187" s="7"/>
       <c r="Q187" s="7"/>
       <c r="R187" s="7">
         <v>0</v>
       </c>
-      <c r="S187" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S187" s="7"/>
       <c r="T187" s="7"/>
       <c r="U187" s="7"/>
       <c r="V187" s="7"/>
       <c r="W187" s="7"/>
       <c r="X187" s="7"/>
-      <c r="Y187" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="Y187" s="7"/>
       <c r="Z187" s="8" t="s">
-        <v>181</v>
+        <v>503</v>
       </c>
       <c r="AA187" s="7" t="s">
         <v>40</v>
@@ -14821,7 +14827,7 @@
         <v>186</v>
       </c>
       <c r="B188" s="3">
-        <v>2026060905</v>
+        <v>2026061283</v>
       </c>
       <c r="C188" s="3">
         <v>1</v>
@@ -14833,16 +14839,16 @@
         <v>345</v>
       </c>
       <c r="F188" s="3" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="G188" s="3" t="s">
-        <v>43</v>
+        <v>303</v>
       </c>
       <c r="H188" s="3" t="s">
-        <v>257</v>
+        <v>315</v>
       </c>
       <c r="I188" s="3" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="J188" s="3"/>
       <c r="K188" s="3"/>
@@ -14850,10 +14856,10 @@
         <v>167</v>
       </c>
       <c r="M188" s="6" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="N188" s="6" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="O188" s="3" t="s">
         <v>39</v>
@@ -14889,7 +14895,7 @@
         <v>187</v>
       </c>
       <c r="B189" s="7">
-        <v>2026060510</v>
+        <v>2026060905</v>
       </c>
       <c r="C189" s="7">
         <v>1</v>
@@ -14898,19 +14904,19 @@
         <v>29</v>
       </c>
       <c r="E189" s="7" t="s">
-        <v>505</v>
+        <v>345</v>
       </c>
       <c r="F189" s="7" t="s">
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="G189" s="7" t="s">
-        <v>506</v>
+        <v>43</v>
       </c>
       <c r="H189" s="7" t="s">
-        <v>507</v>
+        <v>257</v>
       </c>
       <c r="I189" s="7" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="J189" s="7"/>
       <c r="K189" s="7"/>
@@ -14918,10 +14924,10 @@
         <v>167</v>
       </c>
       <c r="M189" s="8" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="N189" s="8" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="O189" s="7" t="s">
         <v>39</v>
@@ -14939,7 +14945,9 @@
       <c r="V189" s="7"/>
       <c r="W189" s="7"/>
       <c r="X189" s="7"/>
-      <c r="Y189" s="7"/>
+      <c r="Y189" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="Z189" s="8" t="s">
         <v>181</v>
       </c>
@@ -14955,7 +14963,7 @@
         <v>188</v>
       </c>
       <c r="B190" s="3">
-        <v>2026060850</v>
+        <v>2026060510</v>
       </c>
       <c r="C190" s="3">
         <v>1</v>
@@ -14964,19 +14972,19 @@
         <v>29</v>
       </c>
       <c r="E190" s="3" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F190" s="3" t="s">
-        <v>113</v>
+        <v>49</v>
       </c>
       <c r="G190" s="3" t="s">
-        <v>164</v>
+        <v>508</v>
       </c>
       <c r="H190" s="3" t="s">
-        <v>165</v>
+        <v>509</v>
       </c>
       <c r="I190" s="3" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="J190" s="3"/>
       <c r="K190" s="3"/>
@@ -14984,10 +14992,10 @@
         <v>167</v>
       </c>
       <c r="M190" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="N190" s="6" t="s">
         <v>512</v>
-      </c>
-      <c r="N190" s="6" t="s">
-        <v>513</v>
       </c>
       <c r="O190" s="3" t="s">
         <v>39</v>
@@ -15001,15 +15009,13 @@
         <v>40</v>
       </c>
       <c r="T190" s="3"/>
-      <c r="U190" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="U190" s="3"/>
       <c r="V190" s="3"/>
       <c r="W190" s="3"/>
       <c r="X190" s="3"/>
       <c r="Y190" s="3"/>
       <c r="Z190" s="6" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="AA190" s="3" t="s">
         <v>40</v>
@@ -15023,7 +15029,7 @@
         <v>189</v>
       </c>
       <c r="B191" s="7">
-        <v>2026060831</v>
+        <v>2026060850</v>
       </c>
       <c r="C191" s="7">
         <v>1</v>
@@ -15032,52 +15038,52 @@
         <v>29</v>
       </c>
       <c r="E191" s="7" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F191" s="7" t="s">
-        <v>87</v>
+        <v>113</v>
       </c>
       <c r="G191" s="7" t="s">
-        <v>237</v>
+        <v>164</v>
       </c>
       <c r="H191" s="7" t="s">
-        <v>303</v>
+        <v>165</v>
       </c>
       <c r="I191" s="7" t="s">
-        <v>514</v>
-      </c>
-      <c r="J191" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="K191" s="7" t="s">
-        <v>197</v>
-      </c>
+        <v>513</v>
+      </c>
+      <c r="J191" s="7"/>
+      <c r="K191" s="7"/>
       <c r="L191" s="8" t="s">
         <v>167</v>
       </c>
       <c r="M191" s="8" t="s">
+        <v>514</v>
+      </c>
+      <c r="N191" s="8" t="s">
         <v>515</v>
       </c>
-      <c r="N191" s="8" t="s">
-        <v>516</v>
-      </c>
       <c r="O191" s="7" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="P191" s="7"/>
       <c r="Q191" s="7"/>
       <c r="R191" s="7">
         <v>0</v>
       </c>
-      <c r="S191" s="7"/>
+      <c r="S191" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T191" s="7"/>
-      <c r="U191" s="7"/>
+      <c r="U191" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="V191" s="7"/>
       <c r="W191" s="7"/>
       <c r="X191" s="7"/>
       <c r="Y191" s="7"/>
       <c r="Z191" s="8" t="s">
-        <v>517</v>
+        <v>170</v>
       </c>
       <c r="AA191" s="7" t="s">
         <v>40</v>
@@ -15091,7 +15097,7 @@
         <v>190</v>
       </c>
       <c r="B192" s="3">
-        <v>2026061529</v>
+        <v>2026060831</v>
       </c>
       <c r="C192" s="3">
         <v>1</v>
@@ -15100,42 +15106,44 @@
         <v>29</v>
       </c>
       <c r="E192" s="3" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F192" s="3" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="G192" s="3" t="s">
-        <v>518</v>
+        <v>237</v>
       </c>
       <c r="H192" s="3" t="s">
-        <v>237</v>
+        <v>303</v>
       </c>
       <c r="I192" s="3" t="s">
-        <v>519</v>
-      </c>
-      <c r="J192" s="3"/>
-      <c r="K192" s="3"/>
+        <v>516</v>
+      </c>
+      <c r="J192" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="K192" s="3" t="s">
+        <v>197</v>
+      </c>
       <c r="L192" s="6" t="s">
         <v>167</v>
       </c>
       <c r="M192" s="6" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="N192" s="6" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="O192" s="3" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="P192" s="3"/>
       <c r="Q192" s="3"/>
       <c r="R192" s="3">
         <v>0</v>
       </c>
-      <c r="S192" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="S192" s="3"/>
       <c r="T192" s="3"/>
       <c r="U192" s="3"/>
       <c r="V192" s="3"/>
@@ -15143,7 +15151,7 @@
       <c r="X192" s="3"/>
       <c r="Y192" s="3"/>
       <c r="Z192" s="6" t="s">
-        <v>181</v>
+        <v>519</v>
       </c>
       <c r="AA192" s="3" t="s">
         <v>40</v>
@@ -15157,7 +15165,7 @@
         <v>191</v>
       </c>
       <c r="B193" s="7">
-        <v>2026061260</v>
+        <v>2026061529</v>
       </c>
       <c r="C193" s="7">
         <v>1</v>
@@ -15166,44 +15174,42 @@
         <v>29</v>
       </c>
       <c r="E193" s="7" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F193" s="7" t="s">
         <v>31</v>
       </c>
       <c r="G193" s="7" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H193" s="7" t="s">
         <v>237</v>
       </c>
       <c r="I193" s="7" t="s">
-        <v>519</v>
-      </c>
-      <c r="J193" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="K193" s="7" t="s">
-        <v>197</v>
-      </c>
+        <v>521</v>
+      </c>
+      <c r="J193" s="7"/>
+      <c r="K193" s="7"/>
       <c r="L193" s="8" t="s">
         <v>167</v>
       </c>
       <c r="M193" s="8" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="N193" s="8" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="O193" s="7" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="P193" s="7"/>
       <c r="Q193" s="7"/>
       <c r="R193" s="7">
         <v>0</v>
       </c>
-      <c r="S193" s="7"/>
+      <c r="S193" s="7" t="s">
+        <v>40</v>
+      </c>
       <c r="T193" s="7"/>
       <c r="U193" s="7"/>
       <c r="V193" s="7"/>
@@ -15211,19 +15217,21 @@
       <c r="X193" s="7"/>
       <c r="Y193" s="7"/>
       <c r="Z193" s="8" t="s">
-        <v>522</v>
+        <v>181</v>
       </c>
       <c r="AA193" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB193" s="7"/>
+      <c r="AB193" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="194" spans="1:28">
       <c r="A194" s="3">
         <v>192</v>
       </c>
       <c r="B194" s="3">
-        <v>2026060149</v>
+        <v>2026061260</v>
       </c>
       <c r="C194" s="3">
         <v>1</v>
@@ -15232,19 +15240,19 @@
         <v>29</v>
       </c>
       <c r="E194" s="3" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F194" s="3" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="G194" s="3" t="s">
-        <v>164</v>
+        <v>520</v>
       </c>
       <c r="H194" s="3" t="s">
-        <v>523</v>
+        <v>237</v>
       </c>
       <c r="I194" s="3" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="J194" s="3" t="s">
         <v>196</v>
@@ -15256,10 +15264,10 @@
         <v>167</v>
       </c>
       <c r="M194" s="6" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="N194" s="6" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="O194" s="3" t="s">
         <v>94</v>
@@ -15277,21 +15285,19 @@
       <c r="X194" s="3"/>
       <c r="Y194" s="3"/>
       <c r="Z194" s="6" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="AA194" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB194" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB194" s="3"/>
     </row>
     <row r="195" spans="1:28">
       <c r="A195" s="7">
         <v>193</v>
       </c>
       <c r="B195" s="7">
-        <v>2026060475</v>
+        <v>2026060149</v>
       </c>
       <c r="C195" s="7">
         <v>1</v>
@@ -15300,7 +15306,7 @@
         <v>29</v>
       </c>
       <c r="E195" s="7" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F195" s="7" t="s">
         <v>49</v>
@@ -15309,33 +15315,35 @@
         <v>164</v>
       </c>
       <c r="H195" s="7" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="I195" s="7" t="s">
-        <v>524</v>
-      </c>
-      <c r="J195" s="7"/>
-      <c r="K195" s="7"/>
+        <v>526</v>
+      </c>
+      <c r="J195" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="K195" s="7" t="s">
+        <v>197</v>
+      </c>
       <c r="L195" s="8" t="s">
         <v>167</v>
       </c>
       <c r="M195" s="8" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="N195" s="8" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="O195" s="7" t="s">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="P195" s="7"/>
       <c r="Q195" s="7"/>
       <c r="R195" s="7">
         <v>0</v>
       </c>
-      <c r="S195" s="7" t="s">
-        <v>40</v>
-      </c>
+      <c r="S195" s="7"/>
       <c r="T195" s="7"/>
       <c r="U195" s="7"/>
       <c r="V195" s="7"/>
@@ -15343,19 +15351,21 @@
       <c r="X195" s="7"/>
       <c r="Y195" s="7"/>
       <c r="Z195" s="8" t="s">
-        <v>181</v>
+        <v>529</v>
       </c>
       <c r="AA195" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="AB195" s="7"/>
+      <c r="AB195" s="7">
+        <v>1</v>
+      </c>
     </row>
     <row r="196" spans="1:28">
       <c r="A196" s="3">
         <v>194</v>
       </c>
       <c r="B196" s="3">
-        <v>2026061222</v>
+        <v>2026060475</v>
       </c>
       <c r="C196" s="3">
         <v>1</v>
@@ -15364,44 +15374,42 @@
         <v>29</v>
       </c>
       <c r="E196" s="3" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F196" s="3" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="G196" s="3" t="s">
-        <v>106</v>
+        <v>164</v>
       </c>
       <c r="H196" s="3" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="I196" s="3" t="s">
-        <v>529</v>
-      </c>
-      <c r="J196" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="K196" s="3" t="s">
-        <v>197</v>
-      </c>
+        <v>526</v>
+      </c>
+      <c r="J196" s="3"/>
+      <c r="K196" s="3"/>
       <c r="L196" s="6" t="s">
         <v>167</v>
       </c>
       <c r="M196" s="6" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="N196" s="6" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="O196" s="3" t="s">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="P196" s="3"/>
       <c r="Q196" s="3"/>
       <c r="R196" s="3">
         <v>0</v>
       </c>
-      <c r="S196" s="3"/>
+      <c r="S196" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="T196" s="3"/>
       <c r="U196" s="3"/>
       <c r="V196" s="3"/>
@@ -15409,21 +15417,19 @@
       <c r="X196" s="3"/>
       <c r="Y196" s="3"/>
       <c r="Z196" s="6" t="s">
-        <v>532</v>
+        <v>181</v>
       </c>
       <c r="AA196" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AB196" s="3">
-        <v>1</v>
-      </c>
+      <c r="AB196" s="3"/>
     </row>
     <row r="197" spans="1:28">
       <c r="A197" s="7">
         <v>195</v>
       </c>
       <c r="B197" s="7">
-        <v>2026061172</v>
+        <v>2026061222</v>
       </c>
       <c r="C197" s="7">
         <v>1</v>
@@ -15432,34 +15438,34 @@
         <v>29</v>
       </c>
       <c r="E197" s="7" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F197" s="7" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="G197" s="7" t="s">
-        <v>70</v>
+        <v>106</v>
       </c>
       <c r="H197" s="7" t="s">
+        <v>530</v>
+      </c>
+      <c r="I197" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="J197" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="K197" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="L197" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="M197" s="8" t="s">
+        <v>532</v>
+      </c>
+      <c r="N197" s="8" t="s">
         <v>533</v>
-      </c>
-      <c r="I197" s="7" t="s">
-        <v>534</v>
-      </c>
-      <c r="J197" s="7" t="s">
-        <v>535</v>
-      </c>
-      <c r="K197" s="7" t="s">
-        <v>536</v>
-      </c>
-      <c r="L197" s="8" t="s">
-        <v>537</v>
-      </c>
-      <c r="M197" s="8" t="s">
-        <v>538</v>
-      </c>
-      <c r="N197" s="8" t="s">
-        <v>539</v>
       </c>
       <c r="O197" s="7" t="s">
         <v>94</v>
@@ -15477,7 +15483,7 @@
       <c r="X197" s="7"/>
       <c r="Y197" s="7"/>
       <c r="Z197" s="8" t="s">
-        <v>540</v>
+        <v>534</v>
       </c>
       <c r="AA197" s="7" t="s">
         <v>40</v>
@@ -15491,7 +15497,7 @@
         <v>196</v>
       </c>
       <c r="B198" s="3">
-        <v>2026061173</v>
+        <v>2026061172</v>
       </c>
       <c r="C198" s="3">
         <v>1</v>
@@ -15500,7 +15506,7 @@
         <v>29</v>
       </c>
       <c r="E198" s="3" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F198" s="3" t="s">
         <v>42</v>
@@ -15509,25 +15515,25 @@
         <v>70</v>
       </c>
       <c r="H198" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="I198" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="J198" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="K198" s="3" t="s">
+        <v>538</v>
+      </c>
+      <c r="L198" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="M198" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="N198" s="6" t="s">
         <v>541</v>
-      </c>
-      <c r="I198" s="3" t="s">
-        <v>542</v>
-      </c>
-      <c r="J198" s="3" t="s">
-        <v>535</v>
-      </c>
-      <c r="K198" s="3" t="s">
-        <v>536</v>
-      </c>
-      <c r="L198" s="6" t="s">
-        <v>537</v>
-      </c>
-      <c r="M198" s="6" t="s">
-        <v>543</v>
-      </c>
-      <c r="N198" s="6" t="s">
-        <v>544</v>
       </c>
       <c r="O198" s="3" t="s">
         <v>94</v>
@@ -15545,47 +15551,115 @@
       <c r="X198" s="3"/>
       <c r="Y198" s="3"/>
       <c r="Z198" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="AA198" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB198" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:28">
+      <c r="A199" s="7">
+        <v>197</v>
+      </c>
+      <c r="B199" s="7">
+        <v>2026061173</v>
+      </c>
+      <c r="C199" s="7">
+        <v>1</v>
+      </c>
+      <c r="D199" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E199" s="7" t="s">
+        <v>507</v>
+      </c>
+      <c r="F199" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G199" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H199" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="I199" s="7" t="s">
+        <v>544</v>
+      </c>
+      <c r="J199" s="7" t="s">
+        <v>537</v>
+      </c>
+      <c r="K199" s="7" t="s">
+        <v>538</v>
+      </c>
+      <c r="L199" s="8" t="s">
+        <v>539</v>
+      </c>
+      <c r="M199" s="8" t="s">
         <v>545</v>
       </c>
-      <c r="AA198" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="AB198" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="199" spans="1:28">
-      <c r="A199" s="9"/>
-      <c r="B199" s="9"/>
-      <c r="C199" s="9"/>
-      <c r="D199" s="9"/>
-      <c r="E199" s="9"/>
-      <c r="F199" s="9"/>
-      <c r="G199" s="9"/>
-      <c r="H199" s="9"/>
-      <c r="I199" s="9"/>
-      <c r="J199" s="9"/>
-      <c r="K199" s="9"/>
-      <c r="L199" s="10"/>
-      <c r="M199" s="10"/>
-      <c r="N199" s="10"/>
-      <c r="O199" s="9"/>
-      <c r="P199" s="9"/>
-      <c r="Q199" s="9"/>
-      <c r="R199" s="9"/>
-      <c r="S199" s="9"/>
-      <c r="T199" s="9"/>
-      <c r="U199" s="9"/>
-      <c r="V199" s="9"/>
-      <c r="W199" s="9"/>
-      <c r="X199" s="9"/>
-      <c r="Y199" s="9"/>
-      <c r="Z199" s="10"/>
-      <c r="AA199" s="9" t="s">
+      <c r="N199" s="8" t="s">
         <v>546</v>
       </c>
-      <c r="AB199" s="9">
-        <v>119</v>
+      <c r="O199" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="P199" s="7"/>
+      <c r="Q199" s="7"/>
+      <c r="R199" s="7">
+        <v>0</v>
+      </c>
+      <c r="S199" s="7"/>
+      <c r="T199" s="7"/>
+      <c r="U199" s="7"/>
+      <c r="V199" s="7"/>
+      <c r="W199" s="7"/>
+      <c r="X199" s="7"/>
+      <c r="Y199" s="7"/>
+      <c r="Z199" s="8" t="s">
+        <v>547</v>
+      </c>
+      <c r="AA199" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB199" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:28">
+      <c r="A200" s="9"/>
+      <c r="B200" s="9"/>
+      <c r="C200" s="9"/>
+      <c r="D200" s="9"/>
+      <c r="E200" s="9"/>
+      <c r="F200" s="9"/>
+      <c r="G200" s="9"/>
+      <c r="H200" s="9"/>
+      <c r="I200" s="9"/>
+      <c r="J200" s="9"/>
+      <c r="K200" s="9"/>
+      <c r="L200" s="10"/>
+      <c r="M200" s="10"/>
+      <c r="N200" s="10"/>
+      <c r="O200" s="9"/>
+      <c r="P200" s="9"/>
+      <c r="Q200" s="9"/>
+      <c r="R200" s="9"/>
+      <c r="S200" s="9"/>
+      <c r="T200" s="9"/>
+      <c r="U200" s="9"/>
+      <c r="V200" s="9"/>
+      <c r="W200" s="9"/>
+      <c r="X200" s="9"/>
+      <c r="Y200" s="9"/>
+      <c r="Z200" s="10"/>
+      <c r="AA200" s="9" t="s">
+        <v>548</v>
+      </c>
+      <c r="AB200" s="9">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>